<commit_message>
Did more editing of assembly instructions.
</commit_message>
<xml_diff>
--- a/parts/spider_dropper_parts.xlsx
+++ b/parts/spider_dropper_parts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github_projects\spider_dropper\parts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{860F9A35-875B-471C-92C8-6FFC5F09EB75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4596E81-7FFA-4A63-B51E-E3EAEAAB9069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10971" yWindow="583" windowWidth="19852" windowHeight="15711" xr2:uid="{92CA6418-27FC-4AD5-98BD-397EC845101D}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18120" xr2:uid="{92CA6418-27FC-4AD5-98BD-397EC845101D}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="107">
   <si>
     <t>Price</t>
   </si>
@@ -61,9 +61,6 @@
     <t>https://monsterguts.com/products/mini-motor-5rpm-110vac</t>
   </si>
   <si>
-    <t>zip ties</t>
-  </si>
-  <si>
     <t>https://www.amazon.com/gp/product/B09NPKBTHR/</t>
   </si>
   <si>
@@ -241,30 +238,9 @@
     <t>power connector</t>
   </si>
   <si>
-    <t>https://www.digikey.com/en/products/detail/same-sky-formerly-cui-devices/PJ-102AH/408448</t>
-  </si>
-  <si>
-    <t>screw terminal</t>
-  </si>
-  <si>
-    <t>2N3904 NPN transistor</t>
-  </si>
-  <si>
     <t>https://www.digikey.com/en/products/detail/central-semiconductor-corp/2N3904-PBFREE/4806876</t>
   </si>
   <si>
-    <t>https://www.digikey.com/en/products/detail/same-sky-formerly-cui-devices/TB007-508-02BE/10064127</t>
-  </si>
-  <si>
-    <t>TIP 120 Darlington transistor</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/stmicroelectronics/TIP120/603564</t>
-  </si>
-  <si>
-    <t>resistors</t>
-  </si>
-  <si>
     <t>https://www.digikey.com/en/products/detail/yageo/CFR-25JB-52-330R/1636</t>
   </si>
   <si>
@@ -274,12 +250,6 @@
     <t>https://www.digikey.com/en/products/detail/honeywell-sensing-and-productivity-solutions/ZX40E30C01/2748598</t>
   </si>
   <si>
-    <t>pin header sockets</t>
-  </si>
-  <si>
-    <t>1N4001 diode</t>
-  </si>
-  <si>
     <t>https://www.digikey.com/en/products/detail/diotec-semiconductor/1N4001/13164614</t>
   </si>
   <si>
@@ -295,15 +265,9 @@
     <t>Amazon shipping is free with Prime.</t>
   </si>
   <si>
-    <t>https://www.digikey.com/en/products/detail/adam-tech/RS1-03-G/9832055</t>
-  </si>
-  <si>
     <t>Slightly Smarter Upgrade</t>
   </si>
   <si>
-    <t>M3 hex nuts</t>
-  </si>
-  <si>
     <t>https://www.amazon.com/gp/product/B0CTQ36QMW/</t>
   </si>
   <si>
@@ -319,9 +283,6 @@
     <t>fishing wire for hanging</t>
   </si>
   <si>
-    <t>In bulk, cable ties are essentially free.</t>
-  </si>
-  <si>
     <t>The DC version (including the Slightly Smarter upgrade) requires a 12VDC power supply.</t>
   </si>
   <si>
@@ -329,6 +290,63 @@
   </si>
   <si>
     <t>The power connector and screw terminal could be omitted in favor of directly wiring pigtail power connectors to the PCB.</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/dp/B0768V9V5Q/</t>
+  </si>
+  <si>
+    <t>3-pin JST XH wire-to-board</t>
+  </si>
+  <si>
+    <t>IRLZ34NPBF</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/jst-sales-america-inc/B3B-XH-A/1651046</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/same-sky-formerly-cui-devices/PJ-044AH/1644569</t>
+  </si>
+  <si>
+    <t>1N4001 diode (or 1N4148)</t>
+  </si>
+  <si>
+    <t>M3 square nuts</t>
+  </si>
+  <si>
+    <t>M3Sx4.0</t>
+  </si>
+  <si>
+    <t>resistor</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/dp/B0CL9MGC82/</t>
+  </si>
+  <si>
+    <t>JST XH female pins</t>
+  </si>
+  <si>
+    <t>3-conductor jacketed cable</t>
+  </si>
+  <si>
+    <t>PG7 cable glands</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/ARTGEAR-Waterproof-Adjustable-Connector-Protector/dp/B07JH2LPZF/</t>
+  </si>
+  <si>
+    <t>JST XH 3-pin housing</t>
+  </si>
+  <si>
+    <t>2-pin JST XH pigtails w/connector</t>
+  </si>
+  <si>
+    <t>In bulk, cable ties are essentially free. Sunk cost on heat-shrink tubing, solder, hot glue.</t>
+  </si>
+  <si>
+    <t>4" zip ties</t>
+  </si>
+  <si>
+    <t>8" zip ties</t>
   </si>
 </sst>
 </file>
@@ -720,7 +738,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A49C792C-E920-409F-B110-1A72354C03E4}">
-  <dimension ref="A1:P53"/>
+  <dimension ref="A1:P62"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="28.3828125" customWidth="1"/>
@@ -736,16 +754,16 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.4">
@@ -753,19 +771,19 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>1</v>
@@ -779,41 +797,41 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B4" s="1">
-        <v>11.99</v>
+        <v>6.99</v>
       </c>
       <c r="C4">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E4" s="1">
         <f>B4*0.1075</f>
-        <v>1.2889250000000001</v>
+        <v>0.75142500000000001</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1">
         <f>B4+E4+F4</f>
-        <v>13.278925000000001</v>
+        <v>7.7414250000000004</v>
       </c>
       <c r="H4" s="1">
         <f>IF(C4&gt;0, G4/C4, 0)</f>
-        <v>3.3197312500000002</v>
+        <v>0.96767812500000006</v>
       </c>
       <c r="I4">
         <v>1</v>
       </c>
       <c r="J4" s="1">
         <f>H4*I4</f>
-        <v>3.3197312500000002</v>
+        <v>0.96767812500000006</v>
       </c>
       <c r="O4" t="s">
         <v>6</v>
@@ -821,36 +839,36 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B5" s="1">
-        <v>11.99</v>
+        <v>22.79</v>
       </c>
       <c r="C5">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E5" s="1">
-        <f t="shared" ref="E5:E8" si="0">B5*0.1075</f>
-        <v>1.2889250000000001</v>
+        <f t="shared" ref="E5:E9" si="0">B5*0.1075</f>
+        <v>2.4499249999999999</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1">
-        <f t="shared" ref="G5:G8" si="1">B5+E5+F5</f>
-        <v>13.278925000000001</v>
+        <f t="shared" ref="G5:G9" si="1">B5+E5+F5</f>
+        <v>25.239924999999999</v>
       </c>
       <c r="H5" s="1">
-        <f t="shared" ref="H5:H8" si="2">IF(C5&gt;0, G5/C5, 0)</f>
-        <v>0.44263083333333336</v>
+        <f t="shared" ref="H5:H9" si="2">IF(C5&gt;0, G5/C5, 0)</f>
+        <v>0.25239925000000002</v>
       </c>
       <c r="I5">
         <v>2</v>
       </c>
       <c r="J5" s="1">
         <f>H5*I5</f>
-        <v>0.88526166666666672</v>
+        <v>0.50479850000000004</v>
       </c>
       <c r="O5" t="s">
         <v>7</v>
@@ -858,47 +876,47 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="B6" s="1">
-        <v>6.29</v>
+        <v>5.99</v>
       </c>
       <c r="C6">
         <v>656</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" si="0"/>
-        <v>0.67617499999999997</v>
+        <v>0.64392499999999997</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1">
         <f t="shared" si="1"/>
-        <v>6.9661749999999998</v>
+        <v>6.6339250000000005</v>
       </c>
       <c r="H6" s="1">
         <f t="shared" si="2"/>
-        <v>1.0619169207317073E-2</v>
+        <v>1.0112690548780489E-2</v>
       </c>
       <c r="I6">
         <v>5</v>
       </c>
       <c r="J6" s="1">
         <f>H6*I6</f>
-        <v>5.3095846036585362E-2</v>
+        <v>5.0563452743902441E-2</v>
       </c>
       <c r="O6" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>105</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E7" s="1">
         <f t="shared" si="0"/>
@@ -923,961 +941,1264 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="1">
+        <v>106</v>
+      </c>
+      <c r="D8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="1">
+        <f t="shared" ref="E8" si="3">B8*0.1075</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1">
+        <f t="shared" ref="G8" si="4">B8+E8+F8</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="1">
+        <f t="shared" ref="H8" si="5">IF(C8&gt;0, G8/C8, 0)</f>
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>2</v>
+      </c>
+      <c r="J8" s="1">
+        <f>H8*I8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="1">
         <f>2*35.99</f>
         <v>71.98</v>
       </c>
-      <c r="C8">
+      <c r="C9">
         <v>2000</v>
       </c>
-      <c r="D8" t="s">
-        <v>34</v>
-      </c>
-      <c r="E8" s="1">
+      <c r="D9" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="1">
         <f t="shared" si="0"/>
         <v>7.7378499999999999</v>
       </c>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1">
+      <c r="F9" s="1"/>
+      <c r="G9" s="1">
         <f t="shared" si="1"/>
         <v>79.717849999999999</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H9" s="1">
         <f t="shared" si="2"/>
         <v>3.9858924999999996E-2</v>
       </c>
-      <c r="I8">
-        <v>70</v>
-      </c>
-      <c r="J8" s="1">
-        <f t="shared" ref="J8" si="3">H8*I8</f>
-        <v>2.7901247499999999</v>
-      </c>
-      <c r="O8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="4">
-        <f>SUM(J4:J8)</f>
-        <v>7.0482135127032528</v>
-      </c>
-      <c r="L9" s="1">
-        <f>J9</f>
-        <v>7.0482135127032528</v>
-      </c>
-      <c r="M9" s="1">
-        <f>J9</f>
-        <v>7.0482135127032528</v>
-      </c>
-      <c r="N9" s="1">
-        <f>J9</f>
-        <v>7.0482135127032528</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" ht="15" thickTop="1" x14ac:dyDescent="0.4"/>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.4">
-      <c r="A11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="J11" s="1"/>
-    </row>
+      <c r="I9">
+        <v>105</v>
+      </c>
+      <c r="J9" s="1">
+        <f t="shared" ref="J9" si="6">H9*I9</f>
+        <v>4.1851871249999997</v>
+      </c>
+      <c r="O9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="4">
+        <f>SUM(J4:J9)</f>
+        <v>5.7082272027439025</v>
+      </c>
+      <c r="L10" s="1">
+        <f>J10</f>
+        <v>5.7082272027439025</v>
+      </c>
+      <c r="M10" s="1">
+        <f>J10</f>
+        <v>5.7082272027439025</v>
+      </c>
+      <c r="N10" s="1">
+        <f>J10</f>
+        <v>5.7082272027439025</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="15" thickTop="1" x14ac:dyDescent="0.4"/>
     <row r="12" spans="1:15" x14ac:dyDescent="0.4">
-      <c r="A12" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="1">
-        <v>18.95</v>
-      </c>
-      <c r="C12">
-        <v>1</v>
-      </c>
-      <c r="D12" t="s">
-        <v>32</v>
-      </c>
-      <c r="E12" s="1">
-        <f t="shared" ref="E12:E13" si="4">B12*0.1075</f>
-        <v>2.0371250000000001</v>
-      </c>
-      <c r="F12" s="1">
-        <v>9.5500000000000007</v>
-      </c>
-      <c r="G12" s="1">
-        <f>B12+E12+F12</f>
-        <v>30.537125</v>
-      </c>
-      <c r="H12" s="1">
-        <f>IF(C12&gt;0, G12/C12, 0)</f>
-        <v>30.537125</v>
-      </c>
-      <c r="I12">
-        <v>1</v>
-      </c>
-      <c r="J12" s="1">
-        <f>H12*I12</f>
-        <v>30.537125</v>
-      </c>
-      <c r="O12" t="s">
-        <v>10</v>
-      </c>
+      <c r="A12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="J12" s="1"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="B13" s="1">
-        <v>7.98</v>
+        <v>18.95</v>
       </c>
       <c r="C13">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E13" s="1">
-        <f t="shared" si="4"/>
-        <v>0.85785</v>
-      </c>
-      <c r="F13" s="1"/>
+        <f t="shared" ref="E13:E16" si="7">B13*0.1075</f>
+        <v>2.0371250000000001</v>
+      </c>
+      <c r="F13" s="1">
+        <v>9.5500000000000007</v>
+      </c>
       <c r="G13" s="1">
-        <f t="shared" ref="G13" si="5">B13+E13+F13</f>
-        <v>8.8378499999999995</v>
+        <f>B13+E13+F13</f>
+        <v>30.537125</v>
       </c>
       <c r="H13" s="1">
         <f>IF(C13&gt;0, G13/C13, 0)</f>
-        <v>8.8378499999999999E-2</v>
+        <v>30.537125</v>
       </c>
       <c r="I13">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J13" s="1">
         <f>H13*I13</f>
+        <v>30.537125</v>
+      </c>
+      <c r="O13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="1">
+        <v>7.98</v>
+      </c>
+      <c r="C14">
+        <v>100</v>
+      </c>
+      <c r="D14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="1">
+        <f t="shared" si="7"/>
+        <v>0.85785</v>
+      </c>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1">
+        <f t="shared" ref="G14:G15" si="8">B14+E14+F14</f>
+        <v>8.8378499999999995</v>
+      </c>
+      <c r="H14" s="1">
+        <f>IF(C14&gt;0, G14/C14, 0)</f>
+        <v>8.8378499999999999E-2</v>
+      </c>
+      <c r="I14">
+        <v>4</v>
+      </c>
+      <c r="J14" s="1">
+        <f>H14*I14</f>
         <v>0.35351399999999999</v>
       </c>
-      <c r="O13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="4">
-        <f>SUM(J12:J13)</f>
-        <v>30.890639</v>
-      </c>
-      <c r="L14" s="1">
-        <f>J14</f>
-        <v>30.890639</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" ht="15.45" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="4"/>
-      <c r="L15" s="1"/>
-    </row>
-    <row r="16" spans="1:15" ht="15" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A17" t="s">
+      <c r="O14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="1">
+        <v>5.99</v>
+      </c>
+      <c r="C15">
+        <v>50</v>
+      </c>
+      <c r="D15" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15" s="1">
+        <f t="shared" si="7"/>
+        <v>0.64392499999999997</v>
+      </c>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1">
+        <f t="shared" si="8"/>
+        <v>6.6339250000000005</v>
+      </c>
+      <c r="H15" s="1">
+        <f t="shared" ref="H15" si="9">IF(C15&gt;0, G15/C15, 0)</f>
+        <v>0.1326785</v>
+      </c>
+      <c r="I15">
+        <v>2</v>
+      </c>
+      <c r="J15" s="1">
+        <f>H15*I15</f>
+        <v>0.26535700000000001</v>
+      </c>
+      <c r="O15" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A16" t="s">
+        <v>95</v>
+      </c>
+      <c r="B16" s="1">
+        <v>9.99</v>
+      </c>
+      <c r="C16">
+        <v>100</v>
+      </c>
+      <c r="D16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E16" s="1">
+        <f t="shared" si="7"/>
+        <v>1.073925</v>
+      </c>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1">
+        <f t="shared" ref="G16" si="10">B16+E16+F16</f>
+        <v>11.063925000000001</v>
+      </c>
+      <c r="H16" s="1">
+        <f t="shared" ref="H16" si="11">IF(C16&gt;0, G16/C16, 0)</f>
+        <v>0.11063925000000001</v>
+      </c>
+      <c r="I16">
+        <v>2</v>
+      </c>
+      <c r="J16" s="1">
+        <f>H16*I16</f>
+        <v>0.22127850000000002</v>
+      </c>
+      <c r="O16" s="5"/>
+    </row>
+    <row r="17" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="4">
+        <f>SUM(J13:J16)</f>
+        <v>31.377274500000002</v>
+      </c>
+      <c r="L17" s="1">
+        <f>J17</f>
+        <v>31.377274500000002</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="15.45" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="4"/>
+      <c r="L18" s="1"/>
+    </row>
+    <row r="19" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A20" t="s">
         <v>4</v>
       </c>
-      <c r="B17" s="1">
-        <v>18.989999999999998</v>
-      </c>
-      <c r="C17">
-        <v>2</v>
-      </c>
-      <c r="D17" t="s">
-        <v>32</v>
-      </c>
-      <c r="E17" s="1">
-        <f t="shared" ref="E17:E19" si="6">B17*0.1075</f>
-        <v>2.0414249999999998</v>
-      </c>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1">
-        <f t="shared" ref="G17:G19" si="7">B17+E17+F17</f>
-        <v>21.031424999999999</v>
-      </c>
-      <c r="H17" s="1">
-        <f t="shared" ref="H17:H19" si="8">IF(C17&gt;0, G17/C17, 0)</f>
-        <v>10.515712499999999</v>
-      </c>
-      <c r="I17">
+      <c r="B20" s="1">
+        <v>9.99</v>
+      </c>
+      <c r="C20">
         <v>1</v>
       </c>
-      <c r="J17" s="1">
-        <f>H17*I17</f>
-        <v>10.515712499999999</v>
-      </c>
-      <c r="O17" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="P17" t="s">
+      <c r="D20" t="s">
+        <v>31</v>
+      </c>
+      <c r="E20" s="1">
+        <f t="shared" ref="E20:E23" si="12">B20*0.1075</f>
+        <v>1.073925</v>
+      </c>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1">
+        <f t="shared" ref="G20:G23" si="13">B20+E20+F20</f>
+        <v>11.063925000000001</v>
+      </c>
+      <c r="H20" s="1">
+        <f t="shared" ref="H20:H23" si="14">IF(C20&gt;0, G20/C20, 0)</f>
+        <v>11.063925000000001</v>
+      </c>
+      <c r="I20">
+        <v>1</v>
+      </c>
+      <c r="J20" s="1">
+        <f>H20*I20</f>
+        <v>11.063925000000001</v>
+      </c>
+      <c r="O20" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="P20" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A18" t="s">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A21" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="1">
-        <v>9.49</v>
-      </c>
-      <c r="C18">
-        <v>10</v>
-      </c>
-      <c r="D18" t="s">
-        <v>32</v>
-      </c>
-      <c r="E18" s="1">
-        <f t="shared" si="6"/>
-        <v>1.0201750000000001</v>
-      </c>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1">
-        <f t="shared" si="7"/>
-        <v>10.510175</v>
-      </c>
-      <c r="H18" s="1">
-        <f t="shared" si="8"/>
-        <v>1.0510174999999999</v>
-      </c>
-      <c r="I18">
+      <c r="B21" s="1">
+        <v>9.89</v>
+      </c>
+      <c r="C21">
+        <v>20</v>
+      </c>
+      <c r="D21" t="s">
+        <v>31</v>
+      </c>
+      <c r="E21" s="1">
+        <f t="shared" si="12"/>
+        <v>1.063175</v>
+      </c>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1">
+        <f t="shared" si="13"/>
+        <v>10.953175</v>
+      </c>
+      <c r="H21" s="1">
+        <f t="shared" si="14"/>
+        <v>0.54765874999999997</v>
+      </c>
+      <c r="I21">
         <v>1</v>
       </c>
-      <c r="J18" s="1">
-        <f>H18*I18</f>
-        <v>1.0510174999999999</v>
-      </c>
-      <c r="O18" t="s">
+      <c r="J21" s="1">
+        <f>H21*I21</f>
+        <v>0.54765874999999997</v>
+      </c>
+      <c r="O21" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A19" t="s">
-        <v>14</v>
-      </c>
-      <c r="B19" s="1">
+      <c r="P21" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A22" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22" s="1">
         <v>5.99</v>
       </c>
-      <c r="C19">
+      <c r="C22">
         <v>50</v>
       </c>
-      <c r="D19" t="s">
-        <v>32</v>
-      </c>
-      <c r="E19" s="1">
-        <f t="shared" si="6"/>
+      <c r="D22" t="s">
+        <v>31</v>
+      </c>
+      <c r="E22" s="1">
+        <f t="shared" si="12"/>
         <v>0.64392499999999997</v>
       </c>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1">
-        <f t="shared" si="7"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1">
+        <f t="shared" si="13"/>
         <v>6.6339250000000005</v>
       </c>
-      <c r="H19" s="1">
-        <f t="shared" si="8"/>
+      <c r="H22" s="1">
+        <f t="shared" si="14"/>
         <v>0.1326785</v>
       </c>
-      <c r="I19">
-        <v>5</v>
-      </c>
-      <c r="J19" s="1">
-        <f>H19*I19</f>
-        <v>0.66339250000000005</v>
-      </c>
-      <c r="O19" s="5" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="4">
-        <f>SUM(J17:J19)</f>
-        <v>12.2301225</v>
-      </c>
-      <c r="M20" s="1">
-        <f>J20</f>
-        <v>12.2301225</v>
-      </c>
-      <c r="N20" s="1">
-        <f>J20</f>
-        <v>12.2301225</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" ht="15.45" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="4"/>
-    </row>
-    <row r="22" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="2" t="s">
-        <v>90</v>
+      <c r="I22">
+        <v>1</v>
+      </c>
+      <c r="J22" s="1">
+        <f>H22*I22</f>
+        <v>0.1326785</v>
+      </c>
+      <c r="O22" s="5" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
-        <v>66</v>
+        <v>95</v>
       </c>
       <c r="B23" s="1">
-        <v>5</v>
+        <v>9.99</v>
       </c>
       <c r="C23">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="D23" t="s">
-        <v>32</v>
-      </c>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1">
-        <v>19.98</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="E23" s="1">
+        <f t="shared" si="12"/>
+        <v>1.073925</v>
+      </c>
+      <c r="F23" s="1"/>
       <c r="G23" s="1">
-        <f t="shared" ref="G23:G26" si="9">B23+E23+F23</f>
-        <v>24.98</v>
+        <f t="shared" si="13"/>
+        <v>11.063925000000001</v>
       </c>
       <c r="H23" s="1">
-        <f t="shared" ref="H23:H26" si="10">IF(C23&gt;0, G23/C23, 0)</f>
-        <v>4.9960000000000004</v>
+        <f t="shared" si="14"/>
+        <v>0.11063925000000001</v>
       </c>
       <c r="I23">
         <v>1</v>
       </c>
       <c r="J23" s="1">
-        <f t="shared" ref="J23:J33" si="11">H23*I23</f>
-        <v>4.9960000000000004</v>
-      </c>
-      <c r="O23" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A24" t="s">
-        <v>85</v>
-      </c>
-      <c r="B24" s="1">
-        <v>15.99</v>
-      </c>
-      <c r="C24">
-        <v>10</v>
-      </c>
-      <c r="D24" t="s">
-        <v>32</v>
-      </c>
-      <c r="E24" s="1">
-        <f t="shared" ref="E24" si="12">B24*0.1075</f>
-        <v>1.718925</v>
-      </c>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1">
-        <f t="shared" ref="G24" si="13">B24+E24+F24</f>
-        <v>17.708925000000001</v>
-      </c>
-      <c r="H24" s="1">
-        <f t="shared" ref="H24" si="14">IF(C24&gt;0, G24/C24, 0)</f>
-        <v>1.7708925</v>
-      </c>
-      <c r="I24">
-        <v>1</v>
-      </c>
-      <c r="J24" s="1">
-        <f t="shared" si="11"/>
-        <v>1.7708925</v>
-      </c>
-      <c r="O24" s="5" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A25" t="s">
-        <v>68</v>
-      </c>
-      <c r="B25" s="1">
-        <v>2.14</v>
-      </c>
-      <c r="C25">
-        <v>10</v>
-      </c>
-      <c r="D25" t="s">
-        <v>32</v>
-      </c>
-      <c r="E25" s="1">
-        <f t="shared" ref="E25:E26" si="15">B25*0.1075</f>
-        <v>0.23005</v>
-      </c>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1">
-        <f t="shared" si="9"/>
-        <v>2.37005</v>
-      </c>
-      <c r="H25" s="1">
-        <f t="shared" si="10"/>
-        <v>0.23700499999999999</v>
-      </c>
-      <c r="I25">
-        <v>1</v>
-      </c>
-      <c r="J25" s="1">
-        <f t="shared" si="11"/>
-        <v>0.23700499999999999</v>
-      </c>
-      <c r="O25" s="5" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A26" t="s">
-        <v>70</v>
-      </c>
-      <c r="B26" s="1">
-        <v>6.2</v>
-      </c>
-      <c r="C26">
-        <v>10</v>
-      </c>
-      <c r="D26" t="s">
-        <v>32</v>
-      </c>
-      <c r="E26" s="1">
-        <f t="shared" si="15"/>
-        <v>0.66649999999999998</v>
-      </c>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1">
-        <f t="shared" si="9"/>
-        <v>6.8665000000000003</v>
-      </c>
-      <c r="H26" s="1">
-        <f t="shared" si="10"/>
-        <v>0.68664999999999998</v>
-      </c>
-      <c r="I26">
-        <v>1</v>
-      </c>
-      <c r="J26" s="1">
-        <f t="shared" si="11"/>
-        <v>0.68664999999999998</v>
-      </c>
-      <c r="O26" t="s">
-        <v>71</v>
+        <f>H23*I23</f>
+        <v>0.11063925000000001</v>
+      </c>
+      <c r="O23" s="5"/>
+    </row>
+    <row r="24" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A24" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="4">
+        <f>SUM(J20:J23)</f>
+        <v>11.854901500000002</v>
+      </c>
+      <c r="M24" s="1">
+        <f>J24</f>
+        <v>11.854901500000002</v>
+      </c>
+      <c r="N24" s="1">
+        <f>J24</f>
+        <v>11.854901500000002</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="15.45" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A25" s="3"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="4"/>
+    </row>
+    <row r="26" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="2" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="B27" s="1">
-        <v>4.01</v>
+        <v>5</v>
       </c>
       <c r="C27">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D27" t="s">
-        <v>32</v>
-      </c>
-      <c r="E27" s="1">
-        <f t="shared" ref="E27" si="16">B27*0.1075</f>
-        <v>0.43107499999999999</v>
-      </c>
-      <c r="F27" s="1"/>
+        <v>31</v>
+      </c>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1">
+        <v>19.98</v>
+      </c>
       <c r="G27" s="1">
-        <f t="shared" ref="G27" si="17">B27+E27+F27</f>
-        <v>4.4410749999999997</v>
+        <f t="shared" ref="G27:G30" si="15">B27+E27+F27</f>
+        <v>24.98</v>
       </c>
       <c r="H27" s="1">
-        <f t="shared" ref="H27" si="18">IF(C27&gt;0, G27/C27, 0)</f>
-        <v>0.44410749999999999</v>
+        <f t="shared" ref="H27:H30" si="16">IF(C27&gt;0, G27/C27, 0)</f>
+        <v>4.9960000000000004</v>
       </c>
       <c r="I27">
         <v>1</v>
       </c>
       <c r="J27" s="1">
-        <f t="shared" si="11"/>
-        <v>0.44410749999999999</v>
+        <f t="shared" ref="J27:J36" si="17">H27*I27</f>
+        <v>4.9960000000000004</v>
       </c>
       <c r="O27" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="B28" s="1">
-        <v>2.1</v>
+        <v>17.989999999999998</v>
       </c>
       <c r="C28">
         <v>10</v>
       </c>
       <c r="D28" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E28" s="1">
-        <f t="shared" ref="E28" si="19">B28*0.1075</f>
-        <v>0.22575000000000001</v>
+        <f t="shared" ref="E28" si="18">B28*0.1075</f>
+        <v>1.9339249999999999</v>
       </c>
       <c r="F28" s="1"/>
       <c r="G28" s="1">
-        <f t="shared" ref="G28" si="20">B28+E28+F28</f>
-        <v>2.3257500000000002</v>
+        <f t="shared" ref="G28" si="19">B28+E28+F28</f>
+        <v>19.923924999999997</v>
       </c>
       <c r="H28" s="1">
-        <f t="shared" ref="H28" si="21">IF(C28&gt;0, G28/C28, 0)</f>
-        <v>0.23257500000000003</v>
+        <f t="shared" ref="H28" si="20">IF(C28&gt;0, G28/C28, 0)</f>
+        <v>1.9923924999999998</v>
       </c>
       <c r="I28">
         <v>1</v>
       </c>
       <c r="J28" s="1">
-        <f t="shared" si="11"/>
-        <v>0.23257500000000003</v>
-      </c>
-      <c r="O28" t="s">
-        <v>89</v>
+        <f t="shared" si="17"/>
+        <v>1.9923924999999998</v>
+      </c>
+      <c r="O28" s="5" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="B29" s="1">
-        <v>2.83</v>
+        <v>2.72</v>
       </c>
       <c r="C29">
         <v>10</v>
       </c>
       <c r="D29" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E29" s="1">
-        <f t="shared" ref="E29" si="22">B29*0.1075</f>
-        <v>0.30422500000000002</v>
+        <f t="shared" ref="E29:E30" si="21">B29*0.1075</f>
+        <v>0.29239999999999999</v>
       </c>
       <c r="F29" s="1"/>
       <c r="G29" s="1">
-        <f t="shared" ref="G29" si="23">B29+E29+F29</f>
-        <v>3.1342250000000003</v>
+        <f t="shared" si="15"/>
+        <v>3.0124000000000004</v>
       </c>
       <c r="H29" s="1">
-        <f t="shared" ref="H29" si="24">IF(C29&gt;0, G29/C29, 0)</f>
-        <v>0.31342250000000005</v>
+        <f t="shared" si="16"/>
+        <v>0.30124000000000006</v>
       </c>
       <c r="I29">
         <v>1</v>
       </c>
       <c r="J29" s="1">
-        <f t="shared" si="11"/>
-        <v>0.31342250000000005</v>
-      </c>
-      <c r="O29" t="s">
-        <v>74</v>
+        <f t="shared" si="17"/>
+        <v>0.30124000000000006</v>
+      </c>
+      <c r="O29" s="5" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="B30" s="1">
-        <v>27.04</v>
+        <v>8.19</v>
       </c>
       <c r="C30">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E30" s="1">
-        <f t="shared" ref="E30" si="25">B30*0.1075</f>
-        <v>2.9068000000000001</v>
+        <f t="shared" si="21"/>
+        <v>0.8804249999999999</v>
       </c>
       <c r="F30" s="1"/>
       <c r="G30" s="1">
-        <f t="shared" ref="G30" si="26">B30+E30+F30</f>
-        <v>29.9468</v>
+        <f t="shared" si="15"/>
+        <v>9.0704250000000002</v>
       </c>
       <c r="H30" s="1">
-        <f t="shared" ref="H30" si="27">IF(C30&gt;0, G30/C30, 0)</f>
-        <v>0.59893600000000002</v>
+        <f t="shared" si="16"/>
+        <v>0.90704249999999997</v>
       </c>
       <c r="I30">
         <v>1</v>
       </c>
       <c r="J30" s="1">
-        <f t="shared" si="11"/>
-        <v>0.59893600000000002</v>
+        <f t="shared" si="17"/>
+        <v>0.90704249999999997</v>
       </c>
       <c r="O30" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="B31" s="1">
-        <v>1.33</v>
+        <v>7.99</v>
       </c>
       <c r="C31">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="D31" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E31" s="1">
-        <f t="shared" ref="E31:E32" si="28">B31*0.1075</f>
-        <v>0.14297500000000002</v>
+        <f t="shared" ref="E31" si="22">B31*0.1075</f>
+        <v>0.85892500000000005</v>
       </c>
       <c r="F31" s="1"/>
       <c r="G31" s="1">
-        <f t="shared" ref="G31:G32" si="29">B31+E31+F31</f>
-        <v>1.4729750000000001</v>
+        <f t="shared" ref="G31" si="23">B31+E31+F31</f>
+        <v>8.8489249999999995</v>
       </c>
       <c r="H31" s="1">
-        <f t="shared" ref="H31:H32" si="30">IF(C31&gt;0, G31/C31, 0)</f>
-        <v>2.9459500000000003E-2</v>
+        <f t="shared" ref="H31" si="24">IF(C31&gt;0, G31/C31, 0)</f>
+        <v>1.7697849999999999</v>
       </c>
       <c r="I31">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J31" s="1">
-        <f t="shared" si="11"/>
-        <v>5.8919000000000006E-2</v>
-      </c>
-      <c r="O31" t="s">
-        <v>79</v>
+        <f t="shared" si="17"/>
+        <v>1.7697849999999999</v>
+      </c>
+      <c r="O31" s="5" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B32" s="1">
-        <v>0.55000000000000004</v>
+        <v>1.08</v>
       </c>
       <c r="C32">
         <v>10</v>
       </c>
       <c r="D32" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E32" s="1">
-        <f t="shared" si="28"/>
-        <v>5.9125000000000004E-2</v>
+        <f t="shared" ref="E32" si="25">B32*0.1075</f>
+        <v>0.11610000000000001</v>
       </c>
       <c r="F32" s="1"/>
       <c r="G32" s="1">
-        <f t="shared" si="29"/>
-        <v>0.60912500000000003</v>
+        <f t="shared" ref="G32" si="26">B32+E32+F32</f>
+        <v>1.1961000000000002</v>
       </c>
       <c r="H32" s="1">
-        <f t="shared" si="30"/>
-        <v>6.0912500000000001E-2</v>
+        <f t="shared" ref="H32" si="27">IF(C32&gt;0, G32/C32, 0)</f>
+        <v>0.11961000000000002</v>
       </c>
       <c r="I32">
         <v>1</v>
       </c>
       <c r="J32" s="1">
-        <f t="shared" si="11"/>
-        <v>6.0912500000000001E-2</v>
+        <f t="shared" si="17"/>
+        <v>0.11961000000000002</v>
       </c>
       <c r="O32" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B33" s="1">
-        <v>4.99</v>
+        <v>2.02</v>
       </c>
       <c r="C33">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D33" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E33" s="1">
-        <f t="shared" ref="E33:E35" si="31">B33*0.1075</f>
-        <v>0.53642500000000004</v>
+        <f t="shared" ref="E33" si="28">B33*0.1075</f>
+        <v>0.21715000000000001</v>
       </c>
       <c r="F33" s="1"/>
       <c r="G33" s="1">
-        <f t="shared" ref="G33:G35" si="32">B33+E33+F33</f>
-        <v>5.5264250000000006</v>
+        <f t="shared" ref="G33" si="29">B33+E33+F33</f>
+        <v>2.2371500000000002</v>
       </c>
       <c r="H33" s="1">
-        <f t="shared" ref="H33:H35" si="33">IF(C33&gt;0, G33/C33, 0)</f>
-        <v>0.27632125000000002</v>
+        <f t="shared" ref="H33" si="30">IF(C33&gt;0, G33/C33, 0)</f>
+        <v>0.22371500000000002</v>
       </c>
       <c r="I33">
         <v>1</v>
       </c>
       <c r="J33" s="1">
-        <f t="shared" si="11"/>
-        <v>0.27632125000000002</v>
+        <f t="shared" si="17"/>
+        <v>0.22371500000000002</v>
       </c>
       <c r="O33" t="s">
-        <v>49</v>
-      </c>
-      <c r="P33" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
-        <v>14</v>
+        <v>96</v>
       </c>
       <c r="B34" s="1">
-        <v>5.99</v>
+        <v>1.33</v>
       </c>
       <c r="C34">
         <v>50</v>
       </c>
       <c r="D34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E34" s="1">
-        <f t="shared" si="31"/>
-        <v>0.64392499999999997</v>
+        <f t="shared" ref="E34:E35" si="31">B34*0.1075</f>
+        <v>0.14297500000000002</v>
       </c>
       <c r="F34" s="1"/>
       <c r="G34" s="1">
-        <f t="shared" si="32"/>
-        <v>6.6339250000000005</v>
+        <f t="shared" ref="G34:G35" si="32">B34+E34+F34</f>
+        <v>1.4729750000000001</v>
       </c>
       <c r="H34" s="1">
-        <f t="shared" si="33"/>
-        <v>0.1326785</v>
+        <f t="shared" ref="H34:H35" si="33">IF(C34&gt;0, G34/C34, 0)</f>
+        <v>2.9459500000000003E-2</v>
       </c>
       <c r="I34">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J34" s="1">
-        <f>H34*I34</f>
-        <v>0.26535700000000001</v>
-      </c>
-      <c r="O34" s="5" t="s">
-        <v>92</v>
+        <f t="shared" si="17"/>
+        <v>2.9459500000000003E-2</v>
+      </c>
+      <c r="O34" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B35" s="1">
-        <v>5.49</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="C35">
-        <v>200</v>
+        <v>10</v>
       </c>
       <c r="D35" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E35" s="1">
         <f t="shared" si="31"/>
-        <v>0.59017500000000001</v>
+        <v>5.9125000000000004E-2</v>
       </c>
       <c r="F35" s="1"/>
       <c r="G35" s="1">
         <f t="shared" si="32"/>
-        <v>6.0801750000000006</v>
+        <v>0.60912500000000003</v>
       </c>
       <c r="H35" s="1">
         <f t="shared" si="33"/>
-        <v>3.0400875000000004E-2</v>
+        <v>6.0912500000000001E-2</v>
       </c>
       <c r="I35">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J35" s="1">
-        <f>H35*I35</f>
-        <v>6.0801750000000009E-2</v>
-      </c>
-      <c r="O35" s="5" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
-      <c r="F36" s="3"/>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
-      <c r="I36" s="3"/>
-      <c r="J36" s="4">
-        <f>SUM(J23:J35)</f>
-        <v>10.001900000000001</v>
-      </c>
-      <c r="M36" s="1"/>
-      <c r="N36" s="1">
-        <f>J36</f>
-        <v>10.001900000000001</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="B37" s="1"/>
-      <c r="E37" s="1"/>
+        <f t="shared" si="17"/>
+        <v>6.0912500000000001E-2</v>
+      </c>
+      <c r="O35" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A36" t="s">
+        <v>72</v>
+      </c>
+      <c r="B36" s="1">
+        <v>4.79</v>
+      </c>
+      <c r="C36">
+        <v>20</v>
+      </c>
+      <c r="D36" t="s">
+        <v>31</v>
+      </c>
+      <c r="E36" s="1">
+        <f t="shared" ref="E36:E43" si="34">B36*0.1075</f>
+        <v>0.51492499999999997</v>
+      </c>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1">
+        <f t="shared" ref="G36:G43" si="35">B36+E36+F36</f>
+        <v>5.3049249999999999</v>
+      </c>
+      <c r="H36" s="1">
+        <f t="shared" ref="H36:H43" si="36">IF(C36&gt;0, G36/C36, 0)</f>
+        <v>0.26524625000000002</v>
+      </c>
+      <c r="I36">
+        <v>1</v>
+      </c>
+      <c r="J36" s="1">
+        <f t="shared" si="17"/>
+        <v>0.26524625000000002</v>
+      </c>
+      <c r="O36" t="s">
+        <v>48</v>
+      </c>
+      <c r="P36" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A37" t="s">
+        <v>13</v>
+      </c>
+      <c r="B37" s="1">
+        <v>5.99</v>
+      </c>
+      <c r="C37">
+        <v>50</v>
+      </c>
+      <c r="D37" t="s">
+        <v>31</v>
+      </c>
+      <c r="E37" s="1">
+        <f t="shared" si="34"/>
+        <v>0.64392499999999997</v>
+      </c>
       <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-      <c r="H37" s="1"/>
-      <c r="J37" s="1"/>
-    </row>
-    <row r="38" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B38" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C38" s="3"/>
-      <c r="D38" s="3"/>
-      <c r="E38" s="4"/>
-      <c r="F38" s="4"/>
-      <c r="G38" s="4"/>
-      <c r="H38" s="4"/>
-      <c r="I38" s="3"/>
-      <c r="J38" s="4"/>
-      <c r="K38" s="3"/>
-      <c r="L38" s="4">
-        <f>SUM(L3:L37)</f>
-        <v>37.938852512703249</v>
-      </c>
-      <c r="M38" s="4">
-        <f>SUM(M3:M37)</f>
-        <v>19.278336012703253</v>
-      </c>
-      <c r="N38" s="4">
-        <f>SUM(N3:N37)</f>
-        <v>29.280236012703256</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="B39" s="1"/>
-      <c r="E39" s="1"/>
+      <c r="G37" s="1">
+        <f t="shared" si="35"/>
+        <v>6.6339250000000005</v>
+      </c>
+      <c r="H37" s="1">
+        <f t="shared" si="36"/>
+        <v>0.1326785</v>
+      </c>
+      <c r="I37">
+        <v>1</v>
+      </c>
+      <c r="J37" s="1">
+        <f t="shared" ref="J37:J44" si="37">H37*I37</f>
+        <v>0.1326785</v>
+      </c>
+      <c r="O37" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A38" t="s">
+        <v>94</v>
+      </c>
+      <c r="B38" s="1">
+        <v>7.95</v>
+      </c>
+      <c r="C38">
+        <v>25</v>
+      </c>
+      <c r="D38" t="s">
+        <v>31</v>
+      </c>
+      <c r="E38" s="1">
+        <f t="shared" si="34"/>
+        <v>0.85462499999999997</v>
+      </c>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1">
+        <f t="shared" si="35"/>
+        <v>8.8046249999999997</v>
+      </c>
+      <c r="H38" s="1">
+        <f t="shared" si="36"/>
+        <v>0.35218499999999997</v>
+      </c>
+      <c r="I38">
+        <v>1</v>
+      </c>
+      <c r="J38" s="1">
+        <f t="shared" si="37"/>
+        <v>0.35218499999999997</v>
+      </c>
+      <c r="O38" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A39" t="s">
+        <v>98</v>
+      </c>
+      <c r="B39" s="1">
+        <v>25.83</v>
+      </c>
+      <c r="C39">
+        <v>500</v>
+      </c>
+      <c r="D39" t="s">
+        <v>31</v>
+      </c>
+      <c r="E39" s="1">
+        <f t="shared" si="34"/>
+        <v>2.7767249999999999</v>
+      </c>
       <c r="F39" s="1"/>
-      <c r="G39" s="1"/>
-      <c r="H39" s="1"/>
-      <c r="J39" s="1"/>
+      <c r="G39" s="1">
+        <f t="shared" si="35"/>
+        <v>28.606724999999997</v>
+      </c>
+      <c r="H39" s="1">
+        <f t="shared" si="36"/>
+        <v>5.7213449999999992E-2</v>
+      </c>
+      <c r="I39">
+        <v>3</v>
+      </c>
+      <c r="J39" s="1">
+        <f t="shared" si="37"/>
+        <v>0.17164034999999997</v>
+      </c>
+      <c r="O39" s="5"/>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
-        <v>30</v>
-      </c>
-      <c r="B40" s="1"/>
-      <c r="E40" s="1"/>
+        <v>102</v>
+      </c>
+      <c r="B40" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="C40">
+        <v>10</v>
+      </c>
+      <c r="D40" t="s">
+        <v>31</v>
+      </c>
+      <c r="E40" s="1">
+        <f t="shared" si="34"/>
+        <v>6.9875000000000007E-2</v>
+      </c>
       <c r="F40" s="1"/>
-      <c r="G40" s="1"/>
-      <c r="H40" s="1"/>
-      <c r="J40" s="1"/>
+      <c r="G40" s="1">
+        <f t="shared" si="35"/>
+        <v>0.71987500000000004</v>
+      </c>
+      <c r="H40" s="1">
+        <f t="shared" si="36"/>
+        <v>7.198750000000001E-2</v>
+      </c>
+      <c r="I40">
+        <v>1</v>
+      </c>
+      <c r="J40" s="1">
+        <f t="shared" si="37"/>
+        <v>7.198750000000001E-2</v>
+      </c>
+      <c r="O40" s="5"/>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A41" t="s">
+        <v>99</v>
+      </c>
+      <c r="B41" s="1">
+        <v>29.98</v>
+      </c>
+      <c r="C41">
+        <v>100</v>
+      </c>
+      <c r="D41" t="s">
+        <v>32</v>
+      </c>
+      <c r="E41" s="1">
+        <f t="shared" si="34"/>
+        <v>3.2228500000000002</v>
+      </c>
+      <c r="F41" s="1"/>
+      <c r="G41" s="1">
+        <f t="shared" si="35"/>
+        <v>33.202849999999998</v>
+      </c>
+      <c r="H41" s="1">
+        <f t="shared" si="36"/>
+        <v>0.3320285</v>
+      </c>
+      <c r="I41">
+        <v>4</v>
+      </c>
+      <c r="J41" s="1">
+        <f t="shared" si="37"/>
+        <v>1.328114</v>
+      </c>
+      <c r="O41" s="5"/>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
-        <v>28</v>
+        <v>105</v>
+      </c>
+      <c r="D42" t="s">
+        <v>31</v>
+      </c>
+      <c r="E42" s="1">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="F42" s="1"/>
+      <c r="G42" s="1">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="H42" s="1">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="I42">
+        <v>2</v>
+      </c>
+      <c r="J42" s="1">
+        <f>H42*I42</f>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
-        <v>20</v>
+        <v>106</v>
+      </c>
+      <c r="D43" t="s">
+        <v>31</v>
+      </c>
+      <c r="E43" s="1">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="F43" s="1"/>
+      <c r="G43" s="1">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="H43" s="1">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="I43">
+        <v>2</v>
+      </c>
+      <c r="J43" s="1">
+        <f>H43*I43</f>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A44" s="5"/>
-    </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A45" t="s">
+      <c r="A44" t="s">
+        <v>100</v>
+      </c>
+      <c r="B44" s="1">
+        <v>8.99</v>
+      </c>
+      <c r="C44">
+        <v>50</v>
+      </c>
+      <c r="D44" t="s">
+        <v>31</v>
+      </c>
+      <c r="E44" s="1">
+        <f t="shared" ref="E44" si="38">B44*0.1075</f>
+        <v>0.96642499999999998</v>
+      </c>
+      <c r="F44" s="1"/>
+      <c r="G44" s="1">
+        <f t="shared" ref="G44" si="39">B44+E44+F44</f>
+        <v>9.9564249999999994</v>
+      </c>
+      <c r="H44" s="1">
+        <f t="shared" ref="H44" si="40">IF(C44&gt;0, G44/C44, 0)</f>
+        <v>0.19912849999999999</v>
+      </c>
+      <c r="I44">
+        <v>1</v>
+      </c>
+      <c r="J44" s="1">
+        <f t="shared" si="37"/>
+        <v>0.19912849999999999</v>
+      </c>
+      <c r="O44" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A45" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="4">
+        <f>SUM(J27:J44)</f>
+        <v>12.921137100000003</v>
+      </c>
+      <c r="M45" s="1"/>
+      <c r="N45" s="1">
+        <f>J45</f>
+        <v>12.921137100000003</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="B46" s="1"/>
+      <c r="E46" s="1"/>
+      <c r="F46" s="1"/>
+      <c r="G46" s="1"/>
+      <c r="H46" s="1"/>
+      <c r="J46" s="1"/>
+    </row>
+    <row r="47" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B47" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C47" s="3"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4"/>
+      <c r="G47" s="4"/>
+      <c r="H47" s="4"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="4"/>
+      <c r="K47" s="3"/>
+      <c r="L47" s="4">
+        <f>SUM(L3:L46)</f>
+        <v>37.085501702743905</v>
+      </c>
+      <c r="M47" s="4">
+        <f>SUM(M3:M46)</f>
+        <v>17.563128702743903</v>
+      </c>
+      <c r="N47" s="4">
+        <f>SUM(N3:N46)</f>
+        <v>30.484265802743906</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="B48" s="1"/>
+      <c r="E48" s="1"/>
+      <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
+      <c r="J48" s="1"/>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A49" t="s">
+        <v>29</v>
+      </c>
+      <c r="B49" s="1"/>
+      <c r="E49" s="1"/>
+      <c r="F49" s="1"/>
+      <c r="G49" s="1"/>
+      <c r="H49" s="1"/>
+      <c r="J49" s="1"/>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A51" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A52" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A53" s="5"/>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A54" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A56" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A58" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A60" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A62" t="s">
         <v>87</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A47" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A49" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A51" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A53" t="s">
-        <v>100</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="O24" r:id="rId1" xr:uid="{394BA01E-496A-4B9E-AF12-01E77921BE0E}"/>
-    <hyperlink ref="O25" r:id="rId2" xr:uid="{229E0547-4398-43AE-9042-0D4FDFFB3BD5}"/>
-    <hyperlink ref="O19" r:id="rId3" xr:uid="{59869D84-F75A-42B0-B422-BA8AA8AB692E}"/>
-    <hyperlink ref="O35" r:id="rId4" xr:uid="{ED21D2F4-CBE0-426A-A036-B9B33370EF91}"/>
-    <hyperlink ref="O34" r:id="rId5" xr:uid="{916C30C5-416A-439A-9D92-626717DEB750}"/>
-    <hyperlink ref="O17" r:id="rId6" xr:uid="{D1850C95-FE4D-4651-A768-4D4B82A92A51}"/>
+    <hyperlink ref="O28" r:id="rId1" xr:uid="{394BA01E-496A-4B9E-AF12-01E77921BE0E}"/>
+    <hyperlink ref="O29" r:id="rId2" xr:uid="{229E0547-4398-43AE-9042-0D4FDFFB3BD5}"/>
+    <hyperlink ref="O22" r:id="rId3" xr:uid="{59869D84-F75A-42B0-B422-BA8AA8AB692E}"/>
+    <hyperlink ref="O38" r:id="rId4" xr:uid="{ED21D2F4-CBE0-426A-A036-B9B33370EF91}"/>
+    <hyperlink ref="O37" r:id="rId5" xr:uid="{916C30C5-416A-439A-9D92-626717DEB750}"/>
+    <hyperlink ref="O20" r:id="rId6" xr:uid="{D1850C95-FE4D-4651-A768-4D4B82A92A51}"/>
+    <hyperlink ref="P21" r:id="rId7" xr:uid="{73F810AA-AEFB-4793-A445-E887A5F2B042}"/>
+    <hyperlink ref="O15" r:id="rId8" xr:uid="{77729D2A-4BC1-468B-9C65-EEFB539A2497}"/>
+    <hyperlink ref="O31" r:id="rId9" xr:uid="{0F1AC341-B54F-4D97-9FD8-521B6BC77D29}"/>
+    <hyperlink ref="O44" r:id="rId10" xr:uid="{B4F36DC8-3A21-4F68-940F-E7861222D837}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId7"/>
+  <pageSetup orientation="portrait" r:id="rId11"/>
 </worksheet>
 </file>
 
@@ -1895,40 +2216,40 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" t="s">
         <v>45</v>
       </c>
-      <c r="B3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="F3" t="s">
         <v>52</v>
-      </c>
-      <c r="D3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F3" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C5" s="1">
         <v>1.95</v>
@@ -1939,23 +2260,23 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" t="s">
         <v>59</v>
-      </c>
-      <c r="C8" t="s">
-        <v>60</v>
       </c>
       <c r="F8">
         <v>4</v>
@@ -1963,10 +2284,10 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C9" s="1">
         <v>1.75</v>
@@ -1974,30 +2295,30 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C10" s="1">
         <v>1.33</v>
       </c>
       <c r="D10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E10" s="1">
         <v>0.25</v>
       </c>
       <c r="F10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C11" s="1">
         <v>2.31</v>
@@ -2008,32 +2329,32 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Started updating assembly.md after last change to shaft adapter.
Also includes updates to the parts spreadsheet.
</commit_message>
<xml_diff>
--- a/parts/spider_dropper_parts.xlsx
+++ b/parts/spider_dropper_parts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github_projects\spider_dropper\parts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AF8F470-9F5B-4219-A96A-4A0E4E92E49B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07BB79F3-E7EB-4619-A8EB-7DE50DEBC013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18120" xr2:uid="{92CA6418-27FC-4AD5-98BD-397EC845101D}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="109">
   <si>
     <t>Price</t>
   </si>
@@ -106,9 +106,6 @@
     <t>Tax</t>
   </si>
   <si>
-    <t>https://www.printedsolid.com/collections/prusament/products/prusament-petg-1-75mm-1kg-prusa-galaxy-black</t>
-  </si>
-  <si>
     <t>Unit</t>
   </si>
   <si>
@@ -178,18 +175,12 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>1, 2, 3</t>
-  </si>
-  <si>
     <t>3. DigiKey price requires large quantity.</t>
   </si>
   <si>
     <t>2. Amazon version may not have UL certification.</t>
   </si>
   <si>
-    <t>1. Specs for current capacity of Amazon version don't match.</t>
-  </si>
-  <si>
     <t>ZX40C30C01-ND</t>
   </si>
   <si>
@@ -331,9 +322,6 @@
     <t>• Amazon shipping is free with Prime.</t>
   </si>
   <si>
-    <t>• In bulk, cable ties are essentially free. Sunk cost on heat-shrink tubing, solder, hot glue.</t>
-  </si>
-  <si>
     <t>credit for unneeded pigtail from DC Option</t>
   </si>
   <si>
@@ -347,6 +335,24 @@
   </si>
   <si>
     <t>M3 square nut</t>
+  </si>
+  <si>
+    <t>1, 2</t>
+  </si>
+  <si>
+    <t>1. Specs for current capacity of Amazon version don't match, but project is low current.</t>
+  </si>
+  <si>
+    <t>• Eating the cost on consumables like heat-shrink tubing, solder, hot glue.</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/dp/B0D5M2X835/</t>
+  </si>
+  <si>
+    <t>https://www.printedsolid.com/products/prusament-petg-1-75mm-2kg-jet-black-made-in-usa?variant=40929368244309</t>
+  </si>
+  <si>
+    <t>• Tax on PCBs is based on estimated tariff of 10% of manufacturing and shipping cost per conversation with ChatGPT.</t>
   </si>
 </sst>
 </file>
@@ -423,7 +429,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -436,6 +442,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="1" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -755,7 +764,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P55"/>
+  <dimension ref="A1:P57"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="28.3828125" customWidth="1"/>
@@ -771,12 +780,12 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>0</v>
@@ -785,7 +794,7 @@
         <v>24</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E3" s="7" t="s">
         <v>25</v>
@@ -812,7 +821,7 @@
         <v>13</v>
       </c>
       <c r="N3" s="7" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.4">
@@ -826,7 +835,7 @@
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E4" s="1">
         <f>B4*0.1075</f>
@@ -863,7 +872,7 @@
         <v>100</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E5" s="1">
         <f t="shared" ref="E5:E9" si="0">B5*0.1075</f>
@@ -891,7 +900,7 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B6" s="1">
         <v>5.99</v>
@@ -900,7 +909,7 @@
         <v>656</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" si="0"/>
@@ -923,63 +932,78 @@
         <v>5.0563452743902441E-2</v>
       </c>
       <c r="O6" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>95</v>
+        <v>92</v>
+      </c>
+      <c r="B7" s="1">
+        <v>5.99</v>
+      </c>
+      <c r="C7">
+        <v>1000</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E7" s="1">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.64392499999999997</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>6.6339250000000005</v>
       </c>
       <c r="H7" s="1">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>6.6339250000000006E-3</v>
       </c>
       <c r="I7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7" s="1">
         <f>H7*I7</f>
-        <v>0</v>
+        <v>6.6339250000000006E-3</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>96</v>
+        <v>93</v>
+      </c>
+      <c r="B8" s="1">
+        <v>14.99</v>
+      </c>
+      <c r="C8">
+        <v>1200</v>
       </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E8" s="1">
         <f t="shared" ref="E8" si="3">B8*0.1075</f>
-        <v>0</v>
+        <v>1.6114250000000001</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1">
         <f t="shared" ref="G8" si="4">B8+E8+F8</f>
-        <v>0</v>
+        <v>16.601424999999999</v>
       </c>
       <c r="H8" s="1">
         <f t="shared" ref="H8" si="5">IF(C8&gt;0, G8/C8, 0)</f>
-        <v>0</v>
+        <v>1.3834520833333332E-2</v>
       </c>
       <c r="I8">
         <v>2</v>
       </c>
       <c r="J8" s="1">
         <f>H8*I8</f>
-        <v>0</v>
+        <v>2.7669041666666665E-2</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.4">
@@ -987,37 +1011,36 @@
         <v>19</v>
       </c>
       <c r="B9" s="1">
-        <f>2*35.99</f>
-        <v>71.98</v>
+        <v>49.99</v>
       </c>
       <c r="C9">
         <v>2000</v>
       </c>
       <c r="D9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E9" s="1">
         <f t="shared" si="0"/>
-        <v>7.7378499999999999</v>
+        <v>5.3739249999999998</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="1">
         <f t="shared" si="1"/>
-        <v>79.717849999999999</v>
+        <v>55.363925000000002</v>
       </c>
       <c r="H9" s="1">
         <f t="shared" si="2"/>
-        <v>3.9858924999999996E-2</v>
+        <v>2.7681962500000001E-2</v>
       </c>
       <c r="I9">
         <v>105</v>
       </c>
       <c r="J9" s="1">
         <f t="shared" ref="J9" si="6">H9*I9</f>
-        <v>4.1851871249999997</v>
+        <v>2.9066060624999999</v>
       </c>
       <c r="O9" t="s">
-        <v>26</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.45">
@@ -1034,19 +1057,19 @@
       <c r="I10" s="3"/>
       <c r="J10" s="4">
         <f>SUM(J4:J9)</f>
-        <v>5.7082272027439025</v>
+        <v>4.4639491069105688</v>
       </c>
       <c r="L10" s="1">
         <f>J10</f>
-        <v>5.7082272027439025</v>
+        <v>4.4639491069105688</v>
       </c>
       <c r="M10" s="1">
         <f>J10</f>
-        <v>5.7082272027439025</v>
+        <v>4.4639491069105688</v>
       </c>
       <c r="N10" s="1">
         <f>J10</f>
-        <v>5.7082272027439025</v>
+        <v>4.4639491069105688</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="15" thickTop="1" x14ac:dyDescent="0.4"/>
@@ -1061,7 +1084,7 @@
         <v>24</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>25</v>
@@ -1093,7 +1116,7 @@
         <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E13" s="1">
         <f t="shared" ref="E13:E16" si="7">B13*0.1075</f>
@@ -1132,7 +1155,7 @@
         <v>100</v>
       </c>
       <c r="D14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E14" s="1">
         <f t="shared" si="7"/>
@@ -1169,7 +1192,7 @@
         <v>50</v>
       </c>
       <c r="D15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E15" s="1">
         <f t="shared" si="7"/>
@@ -1192,12 +1215,12 @@
         <v>0.26535700000000001</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B16" s="1">
         <v>9.99</v>
@@ -1206,7 +1229,7 @@
         <v>100</v>
       </c>
       <c r="D16" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E16" s="1">
         <f t="shared" si="7"/>
@@ -1275,7 +1298,7 @@
         <v>24</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>25</v>
@@ -1307,19 +1330,19 @@
         <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E20" s="1">
-        <f t="shared" ref="E20:E23" si="12">B20*0.1075</f>
+        <f t="shared" ref="E20:E24" si="12">B20*0.1075</f>
         <v>1.073925</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1">
-        <f t="shared" ref="G20:G23" si="13">B20+E20+F20</f>
+        <f t="shared" ref="G20:G24" si="13">B20+E20+F20</f>
         <v>11.063925000000001</v>
       </c>
       <c r="H20" s="1">
-        <f t="shared" ref="H20:H23" si="14">IF(C20&gt;0, G20/C20, 0)</f>
+        <f t="shared" ref="H20:H24" si="14">IF(C20&gt;0, G20/C20, 0)</f>
         <v>11.063925000000001</v>
       </c>
       <c r="I20">
@@ -1330,7 +1353,7 @@
         <v>11.063925000000001</v>
       </c>
       <c r="O20" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="P20" t="s">
         <v>5</v>
@@ -1338,7 +1361,7 @@
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B21" s="1">
         <v>9.89</v>
@@ -1347,7 +1370,7 @@
         <v>10</v>
       </c>
       <c r="D21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E21" s="1">
         <f t="shared" si="12"/>
@@ -1373,7 +1396,7 @@
         <v>8</v>
       </c>
       <c r="P21" s="5" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.4">
@@ -1387,7 +1410,7 @@
         <v>50</v>
       </c>
       <c r="D22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E22" s="1">
         <f t="shared" si="12"/>
@@ -1403,19 +1426,19 @@
         <v>0.1326785</v>
       </c>
       <c r="I22">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J22" s="1">
         <f>H22*I22</f>
-        <v>0.1326785</v>
+        <v>0.79607099999999997</v>
       </c>
       <c r="O22" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B23" s="1">
         <v>9.99</v>
@@ -1424,7 +1447,7 @@
         <v>100</v>
       </c>
       <c r="D23" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E23" s="1">
         <f t="shared" si="12"/>
@@ -1448,633 +1471,635 @@
       </c>
       <c r="O23" s="5"/>
     </row>
-    <row r="24" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A24" s="3" t="s">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A24" t="s">
+        <v>92</v>
+      </c>
+      <c r="B24" s="1">
+        <v>5.99</v>
+      </c>
+      <c r="C24">
+        <v>1000</v>
+      </c>
+      <c r="D24" t="s">
+        <v>27</v>
+      </c>
+      <c r="E24" s="1">
+        <f t="shared" si="12"/>
+        <v>0.64392499999999997</v>
+      </c>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1">
+        <f t="shared" si="13"/>
+        <v>6.6339250000000005</v>
+      </c>
+      <c r="H24" s="1">
+        <f t="shared" si="14"/>
+        <v>6.6339250000000006E-3</v>
+      </c>
+      <c r="I24">
+        <v>1</v>
+      </c>
+      <c r="J24" s="1">
+        <f>H24*I24</f>
+        <v>6.6339250000000006E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A25" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="4">
-        <f>SUM(J20:J23)</f>
-        <v>12.402560250000002</v>
-      </c>
-      <c r="M24" s="1">
-        <f>J24</f>
-        <v>12.402560250000002</v>
-      </c>
-      <c r="N24" s="1">
-        <f>J24</f>
-        <v>12.402560250000002</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="8"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
-      <c r="J25" s="9"/>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A26" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B26" s="7" t="s">
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="4">
+        <f>SUM(J20:J24)</f>
+        <v>13.072586675</v>
+      </c>
+      <c r="M25" s="1">
+        <f>J25</f>
+        <v>13.072586675</v>
+      </c>
+      <c r="N25" s="1">
+        <f>J25</f>
+        <v>13.072586675</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="8"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="9"/>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A27" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B27" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C27" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D26" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E26" s="7" t="s">
+      <c r="D27" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E27" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="F27" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="G26" s="7" t="s">
+      <c r="G27" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="H26" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="I26" s="7" t="s">
+      <c r="H27" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="I27" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="J26" s="7" t="s">
+      <c r="J27" s="7" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A27" t="s">
-        <v>62</v>
-      </c>
-      <c r="B27" s="1">
-        <v>5</v>
-      </c>
-      <c r="C27">
-        <v>5</v>
-      </c>
-      <c r="D27" t="s">
-        <v>28</v>
-      </c>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1">
-        <v>19.98</v>
-      </c>
-      <c r="G27" s="1">
-        <f t="shared" ref="G27:G31" si="15">B27+E27+F27</f>
-        <v>24.98</v>
-      </c>
-      <c r="H27" s="1">
-        <f t="shared" ref="H27:H31" si="16">IF(C27&gt;0, G27/C27, 0)</f>
-        <v>4.9960000000000004</v>
-      </c>
-      <c r="I27">
-        <v>1</v>
-      </c>
-      <c r="J27" s="1">
-        <f t="shared" ref="J27:J37" si="17">H27*I27</f>
-        <v>4.9960000000000004</v>
-      </c>
-      <c r="O27" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="B28" s="1">
+        <v>19.48</v>
+      </c>
+      <c r="C28">
+        <v>25</v>
+      </c>
+      <c r="D28" t="s">
+        <v>27</v>
+      </c>
+      <c r="E28" s="1">
+        <f>10%*SUM(B28, F28)</f>
+        <v>4.5190000000000001</v>
+      </c>
+      <c r="F28" s="1">
+        <v>25.71</v>
+      </c>
+      <c r="G28" s="1">
+        <f t="shared" ref="G28:G31" si="15">B28+E28+F28</f>
+        <v>49.709000000000003</v>
+      </c>
+      <c r="H28" s="1">
+        <f t="shared" ref="H28:H31" si="16">IF(C28&gt;0, G28/C28, 0)</f>
+        <v>1.9883600000000001</v>
+      </c>
+      <c r="I28">
+        <v>1</v>
+      </c>
+      <c r="J28" s="1">
+        <f t="shared" ref="J28:J38" si="17">H28*I28</f>
+        <v>1.9883600000000001</v>
+      </c>
+      <c r="O28" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A29" t="s">
+        <v>69</v>
+      </c>
+      <c r="B29" s="1">
         <v>17.989999999999998</v>
       </c>
-      <c r="C28">
+      <c r="C29">
         <v>10</v>
       </c>
-      <c r="D28" t="s">
-        <v>28</v>
-      </c>
-      <c r="E28" s="1">
-        <f t="shared" ref="E28" si="18">B28*0.1075</f>
+      <c r="D29" t="s">
+        <v>27</v>
+      </c>
+      <c r="E29" s="1">
+        <f t="shared" ref="E29" si="18">B29*0.1075</f>
         <v>1.9339249999999999</v>
       </c>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1">
-        <f t="shared" ref="G28" si="19">B28+E28+F28</f>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1">
+        <f t="shared" ref="G29" si="19">B29+E29+F29</f>
         <v>19.923924999999997</v>
       </c>
-      <c r="H28" s="1">
-        <f t="shared" ref="H28" si="20">IF(C28&gt;0, G28/C28, 0)</f>
+      <c r="H29" s="1">
+        <f t="shared" ref="H29" si="20">IF(C29&gt;0, G29/C29, 0)</f>
         <v>1.9923924999999998</v>
       </c>
-      <c r="I28">
-        <v>1</v>
-      </c>
-      <c r="J28" s="1">
+      <c r="I29">
+        <v>1</v>
+      </c>
+      <c r="J29" s="1">
         <f t="shared" si="17"/>
         <v>1.9923924999999998</v>
       </c>
-      <c r="O28" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A29" t="s">
-        <v>64</v>
-      </c>
-      <c r="B29" s="1">
-        <v>2.72</v>
-      </c>
-      <c r="C29">
-        <v>10</v>
-      </c>
-      <c r="D29" t="s">
-        <v>28</v>
-      </c>
-      <c r="E29" s="1">
-        <f t="shared" ref="E29:E31" si="21">B29*0.1075</f>
-        <v>0.29239999999999999</v>
-      </c>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1">
-        <f t="shared" si="15"/>
-        <v>3.0124000000000004</v>
-      </c>
-      <c r="H29" s="1">
-        <f t="shared" si="16"/>
-        <v>0.30124000000000006</v>
-      </c>
-      <c r="I29">
-        <v>1</v>
-      </c>
-      <c r="J29" s="1">
-        <f t="shared" si="17"/>
-        <v>0.30124000000000006</v>
-      </c>
       <c r="O29" s="5" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B30" s="1">
-        <v>8.19</v>
+        <v>2.72</v>
       </c>
       <c r="C30">
         <v>10</v>
       </c>
       <c r="D30" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E30" s="1">
-        <f t="shared" si="21"/>
-        <v>0.8804249999999999</v>
+        <f t="shared" ref="E30:E31" si="21">B30*0.1075</f>
+        <v>0.29239999999999999</v>
       </c>
       <c r="F30" s="1"/>
       <c r="G30" s="1">
         <f t="shared" si="15"/>
-        <v>9.0704250000000002</v>
+        <v>3.0124000000000004</v>
       </c>
       <c r="H30" s="1">
         <f t="shared" si="16"/>
-        <v>0.90704249999999997</v>
+        <v>0.30124000000000006</v>
       </c>
       <c r="I30">
         <v>1</v>
       </c>
       <c r="J30" s="1">
         <f t="shared" si="17"/>
+        <v>0.30124000000000006</v>
+      </c>
+      <c r="O30" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A31" t="s">
+        <v>63</v>
+      </c>
+      <c r="B31" s="1">
+        <v>8.19</v>
+      </c>
+      <c r="C31">
+        <v>10</v>
+      </c>
+      <c r="D31" t="s">
+        <v>27</v>
+      </c>
+      <c r="E31" s="1">
+        <f t="shared" si="21"/>
+        <v>0.8804249999999999</v>
+      </c>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1">
+        <f t="shared" si="15"/>
+        <v>9.0704250000000002</v>
+      </c>
+      <c r="H31" s="1">
+        <f t="shared" si="16"/>
         <v>0.90704249999999997</v>
       </c>
-      <c r="O30" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A31" t="str">
-        <f>A21</f>
+      <c r="I31">
+        <v>1</v>
+      </c>
+      <c r="J31" s="1">
+        <f t="shared" si="17"/>
+        <v>0.90704249999999997</v>
+      </c>
+      <c r="O31" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A32" t="str">
+        <f t="shared" ref="A32:H32" si="22">A21</f>
         <v>DC power pigtail</v>
       </c>
-      <c r="B31" s="1">
-        <f>B21</f>
+      <c r="B32" s="1">
+        <f t="shared" si="22"/>
         <v>9.89</v>
       </c>
-      <c r="C31">
-        <f>C21</f>
+      <c r="C32">
+        <f t="shared" si="22"/>
         <v>10</v>
       </c>
-      <c r="D31" t="str">
-        <f>D21</f>
+      <c r="D32" t="str">
+        <f t="shared" si="22"/>
         <v>count</v>
       </c>
-      <c r="E31" s="1">
-        <f>E21</f>
+      <c r="E32" s="1">
+        <f t="shared" si="22"/>
         <v>1.063175</v>
       </c>
-      <c r="F31" s="1">
-        <f>F21</f>
+      <c r="F32" s="1">
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
-      <c r="G31" s="1">
-        <f>G21</f>
+      <c r="G32" s="1">
+        <f t="shared" si="22"/>
         <v>10.953175</v>
       </c>
-      <c r="H31" s="1">
-        <f>H21</f>
+      <c r="H32" s="1">
+        <f t="shared" si="22"/>
         <v>1.0953174999999999</v>
       </c>
-      <c r="I31">
+      <c r="I32">
         <v>-1</v>
       </c>
-      <c r="J31" s="1">
-        <f>H31*I31</f>
+      <c r="J32" s="1">
+        <f>H32*I32</f>
         <v>-1.0953174999999999</v>
       </c>
-      <c r="O31" t="s">
-        <v>102</v>
-      </c>
-      <c r="P31" s="5"/>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A32" t="s">
-        <v>94</v>
-      </c>
-      <c r="B32" s="1">
+      <c r="O32" t="s">
+        <v>98</v>
+      </c>
+      <c r="P32" s="5"/>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A33" t="s">
+        <v>91</v>
+      </c>
+      <c r="B33" s="1">
         <v>7.99</v>
       </c>
-      <c r="C32">
+      <c r="C33">
         <v>5</v>
       </c>
-      <c r="D32" t="s">
-        <v>28</v>
-      </c>
-      <c r="E32" s="1">
-        <f t="shared" ref="E32" si="22">B32*0.1075</f>
+      <c r="D33" t="s">
+        <v>27</v>
+      </c>
+      <c r="E33" s="1">
+        <f t="shared" ref="E33" si="23">B33*0.1075</f>
         <v>0.85892500000000005</v>
       </c>
-      <c r="F32" s="1"/>
-      <c r="G32" s="1">
-        <f t="shared" ref="G32" si="23">B32+E32+F32</f>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1">
+        <f t="shared" ref="G33" si="24">B33+E33+F33</f>
         <v>8.8489249999999995</v>
       </c>
-      <c r="H32" s="1">
-        <f t="shared" ref="H32" si="24">IF(C32&gt;0, G32/C32, 0)</f>
+      <c r="H33" s="1">
+        <f t="shared" ref="H33" si="25">IF(C33&gt;0, G33/C33, 0)</f>
         <v>1.7697849999999999</v>
       </c>
-      <c r="I32">
-        <v>1</v>
-      </c>
-      <c r="J32" s="1">
+      <c r="I33">
+        <v>1</v>
+      </c>
+      <c r="J33" s="1">
         <f t="shared" si="17"/>
         <v>1.7697849999999999</v>
       </c>
-      <c r="O32" s="5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A33" t="s">
-        <v>82</v>
-      </c>
-      <c r="B33" s="1">
+      <c r="O33" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A34" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34" s="1">
         <v>1.08</v>
       </c>
-      <c r="C33">
+      <c r="C34">
         <v>10</v>
       </c>
-      <c r="D33" t="s">
-        <v>28</v>
-      </c>
-      <c r="E33" s="1">
-        <f t="shared" ref="E33" si="25">B33*0.1075</f>
+      <c r="D34" t="s">
+        <v>27</v>
+      </c>
+      <c r="E34" s="1">
+        <f t="shared" ref="E34" si="26">B34*0.1075</f>
         <v>0.11610000000000001</v>
       </c>
-      <c r="F33" s="1"/>
-      <c r="G33" s="1">
-        <f t="shared" ref="G33" si="26">B33+E33+F33</f>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1">
+        <f t="shared" ref="G34" si="27">B34+E34+F34</f>
         <v>1.1961000000000002</v>
       </c>
-      <c r="H33" s="1">
-        <f t="shared" ref="H33" si="27">IF(C33&gt;0, G33/C33, 0)</f>
+      <c r="H34" s="1">
+        <f t="shared" ref="H34" si="28">IF(C34&gt;0, G34/C34, 0)</f>
         <v>0.11961000000000002</v>
       </c>
-      <c r="I33">
-        <v>1</v>
-      </c>
-      <c r="J33" s="1">
+      <c r="I34">
+        <v>1</v>
+      </c>
+      <c r="J34" s="1">
         <f t="shared" si="17"/>
         <v>0.11961000000000002</v>
       </c>
-      <c r="O33" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A34" t="s">
-        <v>83</v>
-      </c>
-      <c r="B34" s="1">
+      <c r="O34" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A35" t="s">
+        <v>80</v>
+      </c>
+      <c r="B35" s="1">
         <v>2.02</v>
       </c>
-      <c r="C34">
+      <c r="C35">
         <v>10</v>
       </c>
-      <c r="D34" t="s">
-        <v>28</v>
-      </c>
-      <c r="E34" s="1">
-        <f t="shared" ref="E34" si="28">B34*0.1075</f>
+      <c r="D35" t="s">
+        <v>27</v>
+      </c>
+      <c r="E35" s="1">
+        <f t="shared" ref="E35" si="29">B35*0.1075</f>
         <v>0.21715000000000001</v>
       </c>
-      <c r="F34" s="1"/>
-      <c r="G34" s="1">
-        <f t="shared" ref="G34" si="29">B34+E34+F34</f>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1">
+        <f t="shared" ref="G35" si="30">B35+E35+F35</f>
         <v>2.2371500000000002</v>
       </c>
-      <c r="H34" s="1">
-        <f t="shared" ref="H34" si="30">IF(C34&gt;0, G34/C34, 0)</f>
+      <c r="H35" s="1">
+        <f t="shared" ref="H35" si="31">IF(C35&gt;0, G35/C35, 0)</f>
         <v>0.22371500000000002</v>
       </c>
-      <c r="I34">
-        <v>1</v>
-      </c>
-      <c r="J34" s="1">
+      <c r="I35">
+        <v>1</v>
+      </c>
+      <c r="J35" s="1">
         <f t="shared" si="17"/>
         <v>0.22371500000000002</v>
       </c>
-      <c r="O34" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A35" t="s">
-        <v>87</v>
-      </c>
-      <c r="B35" s="1">
+      <c r="O35" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A36" t="s">
+        <v>84</v>
+      </c>
+      <c r="B36" s="1">
         <v>1.33</v>
       </c>
-      <c r="C35">
+      <c r="C36">
         <v>50</v>
       </c>
-      <c r="D35" t="s">
-        <v>28</v>
-      </c>
-      <c r="E35" s="1">
-        <f t="shared" ref="E35:E36" si="31">B35*0.1075</f>
+      <c r="D36" t="s">
+        <v>27</v>
+      </c>
+      <c r="E36" s="1">
+        <f t="shared" ref="E36:E37" si="32">B36*0.1075</f>
         <v>0.14297500000000002</v>
       </c>
-      <c r="F35" s="1"/>
-      <c r="G35" s="1">
-        <f t="shared" ref="G35:G36" si="32">B35+E35+F35</f>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1">
+        <f t="shared" ref="G36:G37" si="33">B36+E36+F36</f>
         <v>1.4729750000000001</v>
       </c>
-      <c r="H35" s="1">
-        <f t="shared" ref="H35:H36" si="33">IF(C35&gt;0, G35/C35, 0)</f>
+      <c r="H36" s="1">
+        <f t="shared" ref="H36:H37" si="34">IF(C36&gt;0, G36/C36, 0)</f>
         <v>2.9459500000000003E-2</v>
       </c>
-      <c r="I35">
-        <v>1</v>
-      </c>
-      <c r="J35" s="1">
+      <c r="I36">
+        <v>1</v>
+      </c>
+      <c r="J36" s="1">
         <f t="shared" si="17"/>
         <v>2.9459500000000003E-2</v>
       </c>
-      <c r="O35" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A36" t="s">
-        <v>86</v>
-      </c>
-      <c r="B36" s="1">
+      <c r="O36" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A37" t="s">
+        <v>83</v>
+      </c>
+      <c r="B37" s="1">
         <v>0.55000000000000004</v>
       </c>
-      <c r="C36">
+      <c r="C37">
         <v>10</v>
       </c>
-      <c r="D36" t="s">
-        <v>28</v>
-      </c>
-      <c r="E36" s="1">
-        <f t="shared" si="31"/>
+      <c r="D37" t="s">
+        <v>27</v>
+      </c>
+      <c r="E37" s="1">
+        <f t="shared" si="32"/>
         <v>5.9125000000000004E-2</v>
       </c>
-      <c r="F36" s="1"/>
-      <c r="G36" s="1">
-        <f t="shared" si="32"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1">
+        <f t="shared" si="33"/>
         <v>0.60912500000000003</v>
       </c>
-      <c r="H36" s="1">
-        <f t="shared" si="33"/>
+      <c r="H37" s="1">
+        <f t="shared" si="34"/>
         <v>6.0912500000000001E-2</v>
       </c>
-      <c r="I36">
-        <v>1</v>
-      </c>
-      <c r="J36" s="1">
+      <c r="I37">
+        <v>1</v>
+      </c>
+      <c r="J37" s="1">
         <f t="shared" si="17"/>
         <v>6.0912500000000001E-2</v>
       </c>
-      <c r="O36" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A37" t="s">
-        <v>69</v>
-      </c>
-      <c r="B37" s="1">
+      <c r="O37" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A38" t="s">
+        <v>66</v>
+      </c>
+      <c r="B38" s="1">
         <v>4.79</v>
       </c>
-      <c r="C37">
+      <c r="C38">
         <v>20</v>
       </c>
-      <c r="D37" t="s">
-        <v>28</v>
-      </c>
-      <c r="E37" s="1">
-        <f t="shared" ref="E37:E44" si="34">B37*0.1075</f>
+      <c r="D38" t="s">
+        <v>27</v>
+      </c>
+      <c r="E38" s="1">
+        <f t="shared" ref="E38:E45" si="35">B38*0.1075</f>
         <v>0.51492499999999997</v>
       </c>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1">
-        <f t="shared" ref="G37:G44" si="35">B37+E37+F37</f>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1">
+        <f t="shared" ref="G38:G45" si="36">B38+E38+F38</f>
         <v>5.3049249999999999</v>
       </c>
-      <c r="H37" s="1">
-        <f t="shared" ref="H37:H44" si="36">IF(C37&gt;0, G37/C37, 0)</f>
+      <c r="H38" s="1">
+        <f t="shared" ref="H38:H45" si="37">IF(C38&gt;0, G38/C38, 0)</f>
         <v>0.26524625000000002</v>
       </c>
-      <c r="I37">
-        <v>1</v>
-      </c>
-      <c r="J37" s="1">
+      <c r="I38">
+        <v>1</v>
+      </c>
+      <c r="J38" s="1">
         <f t="shared" si="17"/>
         <v>0.26524625000000002</v>
       </c>
-      <c r="O37" t="s">
-        <v>45</v>
-      </c>
-      <c r="P37" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A38" t="s">
-        <v>12</v>
-      </c>
-      <c r="B38" s="1">
-        <v>5.99</v>
-      </c>
-      <c r="C38">
-        <v>50</v>
-      </c>
-      <c r="D38" t="s">
-        <v>28</v>
-      </c>
-      <c r="E38" s="1">
-        <f t="shared" si="34"/>
-        <v>0.64392499999999997</v>
-      </c>
-      <c r="F38" s="1"/>
-      <c r="G38" s="1">
-        <f t="shared" si="35"/>
-        <v>6.6339250000000005</v>
-      </c>
-      <c r="H38" s="1">
-        <f t="shared" si="36"/>
-        <v>0.1326785</v>
-      </c>
-      <c r="I38">
-        <v>1</v>
-      </c>
-      <c r="J38" s="1">
-        <f t="shared" ref="J38:J45" si="37">H38*I38</f>
-        <v>0.1326785</v>
-      </c>
-      <c r="O38" s="5" t="s">
-        <v>75</v>
+      <c r="O38" t="s">
+        <v>44</v>
+      </c>
+      <c r="P38" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
-        <v>106</v>
+        <v>12</v>
       </c>
       <c r="B39" s="1">
-        <v>7.95</v>
+        <v>5.99</v>
       </c>
       <c r="C39">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="D39" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E39" s="1">
-        <f t="shared" si="34"/>
-        <v>0.85462499999999997</v>
+        <f t="shared" si="35"/>
+        <v>0.64392499999999997</v>
       </c>
       <c r="F39" s="1"/>
       <c r="G39" s="1">
+        <f t="shared" si="36"/>
+        <v>6.6339250000000005</v>
+      </c>
+      <c r="H39" s="1">
+        <f t="shared" si="37"/>
+        <v>0.1326785</v>
+      </c>
+      <c r="I39">
+        <v>1</v>
+      </c>
+      <c r="J39" s="1">
+        <f t="shared" ref="J39:J46" si="38">H39*I39</f>
+        <v>0.1326785</v>
+      </c>
+      <c r="O39" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A40" t="s">
+        <v>102</v>
+      </c>
+      <c r="B40" s="1">
+        <v>7.95</v>
+      </c>
+      <c r="C40">
+        <v>25</v>
+      </c>
+      <c r="D40" t="s">
+        <v>27</v>
+      </c>
+      <c r="E40" s="1">
         <f t="shared" si="35"/>
+        <v>0.85462499999999997</v>
+      </c>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1">
+        <f t="shared" si="36"/>
         <v>8.8046249999999997</v>
       </c>
-      <c r="H39" s="1">
-        <f t="shared" si="36"/>
-        <v>0.35218499999999997</v>
-      </c>
-      <c r="I39">
-        <v>1</v>
-      </c>
-      <c r="J39" s="1">
+      <c r="H40" s="1">
         <f t="shared" si="37"/>
         <v>0.35218499999999997</v>
       </c>
-      <c r="O39" s="5" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A40" t="s">
-        <v>89</v>
-      </c>
-      <c r="B40" s="1">
-        <v>25.83</v>
-      </c>
-      <c r="C40">
-        <v>500</v>
-      </c>
-      <c r="D40" t="s">
-        <v>28</v>
-      </c>
-      <c r="E40" s="1">
-        <f t="shared" si="34"/>
-        <v>2.7767249999999999</v>
-      </c>
-      <c r="F40" s="1"/>
-      <c r="G40" s="1">
-        <f t="shared" si="35"/>
-        <v>28.606724999999997</v>
-      </c>
-      <c r="H40" s="1">
-        <f t="shared" si="36"/>
-        <v>5.7213449999999992E-2</v>
-      </c>
       <c r="I40">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J40" s="1">
-        <f t="shared" si="37"/>
-        <v>0.17164034999999997</v>
-      </c>
-      <c r="O40" s="5"/>
+        <f t="shared" si="38"/>
+        <v>0.35218499999999997</v>
+      </c>
+      <c r="O40" s="5" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="B41" s="1">
-        <v>0.65</v>
+        <v>25.83</v>
       </c>
       <c r="C41">
-        <v>10</v>
+        <v>500</v>
       </c>
       <c r="D41" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E41" s="1">
-        <f t="shared" si="34"/>
-        <v>6.9875000000000007E-2</v>
+        <f t="shared" si="35"/>
+        <v>2.7767249999999999</v>
       </c>
       <c r="F41" s="1"/>
       <c r="G41" s="1">
-        <f t="shared" si="35"/>
-        <v>0.71987500000000004</v>
+        <f t="shared" si="36"/>
+        <v>28.606724999999997</v>
       </c>
       <c r="H41" s="1">
-        <f t="shared" si="36"/>
-        <v>7.198750000000001E-2</v>
+        <f t="shared" si="37"/>
+        <v>5.7213449999999992E-2</v>
       </c>
       <c r="I41">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J41" s="1">
-        <f t="shared" si="37"/>
-        <v>7.198750000000001E-2</v>
+        <f t="shared" si="38"/>
+        <v>0.17164034999999997</v>
       </c>
       <c r="O41" s="5"/>
     </row>
@@ -2083,206 +2108,242 @@
         <v>90</v>
       </c>
       <c r="B42" s="1">
-        <v>29.98</v>
+        <v>0.65</v>
       </c>
       <c r="C42">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="D42" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E42" s="1">
-        <f t="shared" si="34"/>
-        <v>3.2228500000000002</v>
+        <f t="shared" si="35"/>
+        <v>6.9875000000000007E-2</v>
       </c>
       <c r="F42" s="1"/>
       <c r="G42" s="1">
-        <f t="shared" si="35"/>
-        <v>33.202849999999998</v>
+        <f t="shared" si="36"/>
+        <v>0.71987500000000004</v>
       </c>
       <c r="H42" s="1">
-        <f t="shared" si="36"/>
-        <v>0.3320285</v>
+        <f t="shared" si="37"/>
+        <v>7.198750000000001E-2</v>
       </c>
       <c r="I42">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J42" s="1">
-        <f t="shared" si="37"/>
-        <v>1.328114</v>
+        <f t="shared" si="38"/>
+        <v>7.198750000000001E-2</v>
       </c>
       <c r="O42" s="5"/>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
-        <v>95</v>
+        <v>87</v>
+      </c>
+      <c r="B43" s="1">
+        <v>29.98</v>
+      </c>
+      <c r="C43">
+        <v>100</v>
       </c>
       <c r="D43" t="s">
         <v>28</v>
       </c>
       <c r="E43" s="1">
-        <f t="shared" si="34"/>
-        <v>0</v>
+        <f t="shared" si="35"/>
+        <v>3.2228500000000002</v>
       </c>
       <c r="F43" s="1"/>
       <c r="G43" s="1">
-        <f t="shared" si="35"/>
-        <v>0</v>
+        <f t="shared" si="36"/>
+        <v>33.202849999999998</v>
       </c>
       <c r="H43" s="1">
-        <f t="shared" si="36"/>
-        <v>0</v>
+        <f t="shared" si="37"/>
+        <v>0.3320285</v>
       </c>
       <c r="I43">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J43" s="1">
-        <f>H43*I43</f>
-        <v>0</v>
-      </c>
+        <f t="shared" si="38"/>
+        <v>1.328114</v>
+      </c>
+      <c r="O43" s="5"/>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
-        <v>96</v>
+        <v>92</v>
+      </c>
+      <c r="B44" s="1">
+        <v>5.99</v>
+      </c>
+      <c r="C44">
+        <v>1000</v>
       </c>
       <c r="D44" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E44" s="1">
-        <f t="shared" si="34"/>
-        <v>0</v>
+        <f t="shared" si="35"/>
+        <v>0.64392499999999997</v>
       </c>
       <c r="F44" s="1"/>
       <c r="G44" s="1">
-        <f t="shared" si="35"/>
-        <v>0</v>
+        <f t="shared" si="36"/>
+        <v>6.6339250000000005</v>
       </c>
       <c r="H44" s="1">
-        <f t="shared" si="36"/>
-        <v>0</v>
+        <f t="shared" si="37"/>
+        <v>6.6339250000000006E-3</v>
       </c>
       <c r="I44">
         <v>2</v>
       </c>
       <c r="J44" s="1">
         <f>H44*I44</f>
-        <v>0</v>
+        <v>1.3267850000000001E-2</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B45" s="1">
-        <v>8.99</v>
+        <v>14.99</v>
       </c>
       <c r="C45">
-        <v>50</v>
+        <v>1200</v>
       </c>
       <c r="D45" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E45" s="1">
-        <f t="shared" ref="E45" si="38">B45*0.1075</f>
-        <v>0.96642499999999998</v>
+        <f t="shared" si="35"/>
+        <v>1.6114250000000001</v>
       </c>
       <c r="F45" s="1"/>
       <c r="G45" s="1">
-        <f t="shared" ref="G45" si="39">B45+E45+F45</f>
+        <f t="shared" si="36"/>
+        <v>16.601424999999999</v>
+      </c>
+      <c r="H45" s="1">
+        <f t="shared" si="37"/>
+        <v>1.3834520833333332E-2</v>
+      </c>
+      <c r="I45">
+        <v>1</v>
+      </c>
+      <c r="J45" s="1">
+        <f>H45*I45</f>
+        <v>1.3834520833333332E-2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A46" t="s">
+        <v>88</v>
+      </c>
+      <c r="B46" s="1">
+        <v>8.99</v>
+      </c>
+      <c r="C46">
+        <v>50</v>
+      </c>
+      <c r="D46" t="s">
+        <v>27</v>
+      </c>
+      <c r="E46" s="1">
+        <f t="shared" ref="E46" si="39">B46*0.1075</f>
+        <v>0.96642499999999998</v>
+      </c>
+      <c r="F46" s="1"/>
+      <c r="G46" s="1">
+        <f t="shared" ref="G46" si="40">B46+E46+F46</f>
         <v>9.9564249999999994</v>
       </c>
-      <c r="H45" s="1">
-        <f t="shared" ref="H45" si="40">IF(C45&gt;0, G45/C45, 0)</f>
+      <c r="H46" s="1">
+        <f t="shared" ref="H46" si="41">IF(C46&gt;0, G46/C46, 0)</f>
         <v>0.19912849999999999</v>
       </c>
-      <c r="I45">
-        <v>1</v>
-      </c>
-      <c r="J45" s="1">
-        <f t="shared" si="37"/>
+      <c r="I46">
+        <v>1</v>
+      </c>
+      <c r="J46" s="1">
+        <f t="shared" si="38"/>
         <v>0.19912849999999999</v>
       </c>
-      <c r="O45" s="5" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="46" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A46" s="3" t="s">
+      <c r="O46" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A47" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B46" s="3"/>
-      <c r="C46" s="3"/>
-      <c r="D46" s="3"/>
-      <c r="E46" s="3"/>
-      <c r="F46" s="3"/>
-      <c r="G46" s="3"/>
-      <c r="H46" s="3"/>
-      <c r="I46" s="3"/>
-      <c r="J46" s="4">
-        <f>SUM(J27:J45)</f>
-        <v>11.825819600000003</v>
-      </c>
-      <c r="M46" s="1"/>
-      <c r="N46" s="1">
-        <f>J46</f>
-        <v>11.825819600000003</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="B47" s="1"/>
-      <c r="E47" s="1"/>
-      <c r="F47" s="1"/>
-      <c r="G47" s="1"/>
-      <c r="H47" s="1"/>
-      <c r="J47" s="1"/>
-      <c r="L47" s="7" t="s">
+      <c r="B47" s="3"/>
+      <c r="C47" s="3"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="4">
+        <f>SUM(J28:J46)</f>
+        <v>8.8452819708333319</v>
+      </c>
+      <c r="M47" s="1"/>
+      <c r="N47" s="1">
+        <f>J47</f>
+        <v>8.8452819708333319</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="B48" s="1"/>
+      <c r="E48" s="1"/>
+      <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
+      <c r="J48" s="1"/>
+      <c r="L48" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="M47" s="7" t="s">
+      <c r="M48" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="N47" s="7" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="48" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B48" s="4" t="s">
+      <c r="N48" s="7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B49" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C48" s="3"/>
-      <c r="D48" s="3"/>
-      <c r="E48" s="4"/>
-      <c r="F48" s="4"/>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4"/>
-      <c r="I48" s="3"/>
-      <c r="J48" s="4"/>
-      <c r="K48" s="3"/>
-      <c r="L48" s="4">
-        <f>SUM(L3:L47)</f>
-        <v>37.085501702743905</v>
-      </c>
-      <c r="M48" s="4">
-        <f>SUM(M3:M47)</f>
-        <v>18.110787452743907</v>
-      </c>
-      <c r="N48" s="4">
-        <f>SUM(N3:N47)</f>
-        <v>29.936607052743909</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="B49" s="1"/>
-      <c r="E49" s="1"/>
-      <c r="F49" s="1"/>
-      <c r="G49" s="1"/>
-      <c r="H49" s="1"/>
-      <c r="J49" s="1"/>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A50" t="s">
-        <v>97</v>
-      </c>
+      <c r="C49" s="3"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="4"/>
+      <c r="F49" s="4"/>
+      <c r="G49" s="4"/>
+      <c r="H49" s="4"/>
+      <c r="I49" s="3"/>
+      <c r="J49" s="4"/>
+      <c r="K49" s="3"/>
+      <c r="L49" s="4">
+        <f>SUM(L3:L48)</f>
+        <v>35.841223606910575</v>
+      </c>
+      <c r="M49" s="4">
+        <f>SUM(M3:M48)</f>
+        <v>17.536535781910569</v>
+      </c>
+      <c r="N49" s="4">
+        <f>SUM(N3:N48)</f>
+        <v>26.381817752743899</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.4">
       <c r="B50" s="1"/>
       <c r="E50" s="1"/>
       <c r="F50" s="1"/>
@@ -2290,51 +2351,68 @@
       <c r="H50" s="1"/>
       <c r="J50" s="1"/>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
-        <v>98</v>
-      </c>
-      <c r="G51" t="s">
+        <v>94</v>
+      </c>
+      <c r="B51" s="1"/>
+      <c r="E51" s="1"/>
+      <c r="F51" s="1"/>
+      <c r="G51" s="1"/>
+      <c r="H51" s="1"/>
+      <c r="J51" s="1"/>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A52" t="s">
+        <v>95</v>
+      </c>
+      <c r="G52" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A52" t="s">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A53" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A54" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A55" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A56" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A57" t="s">
         <v>99</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A53" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A54" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A55" t="s">
-        <v>103</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="O28" r:id="rId1" xr:uid="{394BA01E-496A-4B9E-AF12-01E77921BE0E}"/>
-    <hyperlink ref="O29" r:id="rId2" xr:uid="{229E0547-4398-43AE-9042-0D4FDFFB3BD5}"/>
+    <hyperlink ref="O29" r:id="rId1" xr:uid="{394BA01E-496A-4B9E-AF12-01E77921BE0E}"/>
+    <hyperlink ref="O30" r:id="rId2" xr:uid="{229E0547-4398-43AE-9042-0D4FDFFB3BD5}"/>
     <hyperlink ref="O22" r:id="rId3" xr:uid="{59869D84-F75A-42B0-B422-BA8AA8AB692E}"/>
-    <hyperlink ref="O39" r:id="rId4" xr:uid="{ED21D2F4-CBE0-426A-A036-B9B33370EF91}"/>
-    <hyperlink ref="O38" r:id="rId5" xr:uid="{916C30C5-416A-439A-9D92-626717DEB750}"/>
+    <hyperlink ref="O40" r:id="rId4" xr:uid="{ED21D2F4-CBE0-426A-A036-B9B33370EF91}"/>
+    <hyperlink ref="O39" r:id="rId5" xr:uid="{916C30C5-416A-439A-9D92-626717DEB750}"/>
     <hyperlink ref="O20" r:id="rId6" xr:uid="{D1850C95-FE4D-4651-A768-4D4B82A92A51}"/>
     <hyperlink ref="P21" r:id="rId7" xr:uid="{73F810AA-AEFB-4793-A445-E887A5F2B042}"/>
     <hyperlink ref="O15" r:id="rId8" xr:uid="{77729D2A-4BC1-468B-9C65-EEFB539A2497}"/>
-    <hyperlink ref="O32" r:id="rId9" xr:uid="{0F1AC341-B54F-4D97-9FD8-521B6BC77D29}"/>
-    <hyperlink ref="O45" r:id="rId10" xr:uid="{B4F36DC8-3A21-4F68-940F-E7861222D837}"/>
+    <hyperlink ref="O33" r:id="rId9" xr:uid="{0F1AC341-B54F-4D97-9FD8-521B6BC77D29}"/>
+    <hyperlink ref="O46" r:id="rId10" xr:uid="{B4F36DC8-3A21-4F68-940F-E7861222D837}"/>
+    <hyperlink ref="O8" r:id="rId11" xr:uid="{2073394A-9AF9-4AAC-B9F4-A09AB6C33DED}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="62" fitToWidth="0" orientation="landscape" r:id="rId11"/>
+  <pageSetup scale="62" fitToWidth="0" orientation="landscape" r:id="rId12"/>
   <ignoredErrors>
-    <ignoredError sqref="E31 G31:H31" formula="1"/>
+    <ignoredError sqref="E32 G32:H32" formula="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2346,152 +2424,156 @@
   <cols>
     <col min="1" max="1" width="14.15234375" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="13.3046875" customWidth="1"/>
+    <col min="3" max="3" width="11.3046875" customWidth="1"/>
     <col min="4" max="4" width="38.921875" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E3" t="s">
         <v>41</v>
       </c>
-      <c r="B3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="F3" t="s">
         <v>48</v>
-      </c>
-      <c r="D3" t="s">
-        <v>43</v>
-      </c>
-      <c r="E3" t="s">
-        <v>42</v>
-      </c>
-      <c r="F3" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>31</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="F4" s="10"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C5" s="1">
         <v>1.95</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="10">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>33</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="F6" s="10"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>34</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="F7" s="10"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F8">
+        <v>53</v>
+      </c>
+      <c r="F8" s="10">
         <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B9" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C9" s="1">
         <v>1.75</v>
       </c>
+      <c r="F9" s="10"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C10" s="1">
         <v>1.33</v>
       </c>
       <c r="D10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E10" s="1">
         <v>0.25</v>
       </c>
-      <c r="F10" t="s">
-        <v>50</v>
+      <c r="F10" s="10" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C11" s="1">
         <v>2.31</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="10">
         <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15" s="6" t="s">
-        <v>53</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated and corrected quantities, prices, and links for some parts.
</commit_message>
<xml_diff>
--- a/parts/spider_dropper_parts.xlsx
+++ b/parts/spider_dropper_parts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github_projects\spider_dropper\parts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07BB79F3-E7EB-4619-A8EB-7DE50DEBC013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3215064-1F86-4847-AA9A-1424A716C47D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18120" xr2:uid="{92CA6418-27FC-4AD5-98BD-397EC845101D}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="110">
   <si>
     <t>Price</t>
   </si>
@@ -49,9 +49,6 @@
     <t>https://www.amazon.com/gp/product/B08CN5G99M/</t>
   </si>
   <si>
-    <t>https://www.amazon.com/gp/product/B07TWZ7X38/</t>
-  </si>
-  <si>
     <t>https://www.amazon.com/gp/product/B072BXB2Y8/</t>
   </si>
   <si>
@@ -247,9 +244,6 @@
     <t>https://www.amazon.com/gp/product/B0CTQ36QMW/</t>
   </si>
   <si>
-    <t>https://www.amazon.com/dp/B0CMGK8MV9/</t>
-  </si>
-  <si>
     <t>https://www.amazon.com/dp/B0CZQMZDM8/</t>
   </si>
   <si>
@@ -262,9 +256,6 @@
     <t>Stupidly Simple Spider Dropper Parts</t>
   </si>
   <si>
-    <t>https://www.amazon.com/dp/B0768V9V5Q/</t>
-  </si>
-  <si>
     <t>3-pin JST XH wire-to-board</t>
   </si>
   <si>
@@ -353,6 +344,18 @@
   </si>
   <si>
     <t>• Tax on PCBs is based on estimated tariff of 10% of manufacturing and shipping cost per conversation with ChatGPT.</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/Pzsmocn-Connector-Compatible-connection-Internet/dp/B096D849KN/</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/dp/B07SDMC9L9</t>
+  </si>
+  <si>
+    <t>Dupont 3-pin connector w/pins</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/B073ST742Z</t>
   </si>
 </sst>
 </file>
@@ -764,7 +767,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P57"/>
+  <dimension ref="A1:P58"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="28.3828125" customWidth="1"/>
@@ -780,30 +783,30 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>25</v>
-      </c>
       <c r="F3" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H3" s="7" t="s">
         <v>1</v>
@@ -815,18 +818,18 @@
         <v>3</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N3" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B4" s="1">
         <v>6.99</v>
@@ -835,7 +838,7 @@
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E4" s="1">
         <f>B4*0.1075</f>
@@ -863,44 +866,44 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" s="1">
-        <v>22.79</v>
+        <v>17.690000000000001</v>
       </c>
       <c r="C5">
         <v>100</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E5" s="1">
         <f t="shared" ref="E5:E9" si="0">B5*0.1075</f>
-        <v>2.4499249999999999</v>
+        <v>1.901675</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1">
         <f t="shared" ref="G5:G9" si="1">B5+E5+F5</f>
-        <v>25.239924999999999</v>
+        <v>19.591675000000002</v>
       </c>
       <c r="H5" s="1">
         <f t="shared" ref="H5:H9" si="2">IF(C5&gt;0, G5/C5, 0)</f>
-        <v>0.25239925000000002</v>
+        <v>0.19591675000000003</v>
       </c>
       <c r="I5">
         <v>2</v>
       </c>
       <c r="J5" s="1">
         <f>H5*I5</f>
-        <v>0.50479850000000004</v>
-      </c>
-      <c r="O5" t="s">
-        <v>7</v>
+        <v>0.39183350000000006</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B6" s="1">
         <v>5.99</v>
@@ -909,7 +912,7 @@
         <v>656</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" si="0"/>
@@ -932,12 +935,12 @@
         <v>5.0563452743902441E-2</v>
       </c>
       <c r="O6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B7" s="1">
         <v>5.99</v>
@@ -946,7 +949,7 @@
         <v>1000</v>
       </c>
       <c r="D7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E7" s="1">
         <f t="shared" si="0"/>
@@ -971,7 +974,7 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B8" s="1">
         <v>14.99</v>
@@ -980,7 +983,7 @@
         <v>1200</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E8" s="1">
         <f t="shared" ref="E8" si="3">B8*0.1075</f>
@@ -1003,12 +1006,12 @@
         <v>2.7669041666666665E-2</v>
       </c>
       <c r="O8" s="5" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" s="1">
         <v>49.99</v>
@@ -1017,7 +1020,7 @@
         <v>2000</v>
       </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E9" s="1">
         <f t="shared" si="0"/>
@@ -1040,12 +1043,12 @@
         <v>2.9066060624999999</v>
       </c>
       <c r="O9" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -1057,43 +1060,43 @@
       <c r="I10" s="3"/>
       <c r="J10" s="4">
         <f>SUM(J4:J9)</f>
-        <v>4.4639491069105688</v>
+        <v>4.3509841069105697</v>
       </c>
       <c r="L10" s="1">
         <f>J10</f>
-        <v>4.4639491069105688</v>
+        <v>4.3509841069105697</v>
       </c>
       <c r="M10" s="1">
         <f>J10</f>
-        <v>4.4639491069105688</v>
+        <v>4.3509841069105697</v>
       </c>
       <c r="N10" s="1">
         <f>J10</f>
-        <v>4.4639491069105688</v>
+        <v>4.3509841069105697</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="15" thickTop="1" x14ac:dyDescent="0.4"/>
     <row r="12" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>0</v>
       </c>
       <c r="C12" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>25</v>
-      </c>
       <c r="F12" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H12" s="7" t="s">
         <v>1</v>
@@ -1107,7 +1110,7 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B13" s="1">
         <v>18.95</v>
@@ -1116,7 +1119,7 @@
         <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E13" s="1">
         <f t="shared" ref="E13:E16" si="7">B13*0.1075</f>
@@ -1141,12 +1144,12 @@
         <v>30.537125</v>
       </c>
       <c r="O13" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B14" s="1">
         <v>7.98</v>
@@ -1155,7 +1158,7 @@
         <v>100</v>
       </c>
       <c r="D14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E14" s="1">
         <f t="shared" si="7"/>
@@ -1178,12 +1181,12 @@
         <v>0.35351399999999999</v>
       </c>
       <c r="O14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15" s="1">
         <v>5.99</v>
@@ -1192,7 +1195,7 @@
         <v>50</v>
       </c>
       <c r="D15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E15" s="1">
         <f t="shared" si="7"/>
@@ -1215,12 +1218,12 @@
         <v>0.26535700000000001</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B16" s="1">
         <v>9.99</v>
@@ -1229,7 +1232,7 @@
         <v>100</v>
       </c>
       <c r="D16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E16" s="1">
         <f t="shared" si="7"/>
@@ -1255,7 +1258,7 @@
     </row>
     <row r="17" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A17" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -1289,25 +1292,25 @@
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A19" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B19" s="7" t="s">
         <v>0</v>
       </c>
       <c r="C19" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E19" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D19" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>25</v>
-      </c>
       <c r="F19" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H19" s="7" t="s">
         <v>1</v>
@@ -1330,7 +1333,7 @@
         <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E20" s="1">
         <f t="shared" ref="E20:E24" si="12">B20*0.1075</f>
@@ -1353,7 +1356,7 @@
         <v>11.063925000000001</v>
       </c>
       <c r="O20" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="P20" t="s">
         <v>5</v>
@@ -1361,16 +1364,16 @@
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B21" s="1">
         <v>9.89</v>
       </c>
       <c r="C21">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E21" s="1">
         <f t="shared" si="12"/>
@@ -1383,25 +1386,23 @@
       </c>
       <c r="H21" s="1">
         <f t="shared" si="14"/>
-        <v>1.0953174999999999</v>
+        <v>0.54765874999999997</v>
       </c>
       <c r="I21">
         <v>1</v>
       </c>
       <c r="J21" s="1">
         <f>H21*I21</f>
-        <v>1.0953174999999999</v>
+        <v>0.54765874999999997</v>
       </c>
       <c r="O21" t="s">
-        <v>8</v>
-      </c>
-      <c r="P21" s="5" t="s">
-        <v>78</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="P21" s="5"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B22" s="1">
         <v>5.99</v>
@@ -1410,7 +1411,7 @@
         <v>50</v>
       </c>
       <c r="D22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E22" s="1">
         <f t="shared" si="12"/>
@@ -1433,12 +1434,12 @@
         <v>0.79607099999999997</v>
       </c>
       <c r="O22" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B23" s="1">
         <v>9.99</v>
@@ -1447,7 +1448,7 @@
         <v>100</v>
       </c>
       <c r="D23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E23" s="1">
         <f t="shared" si="12"/>
@@ -1473,7 +1474,7 @@
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B24" s="1">
         <v>5.99</v>
@@ -1482,7 +1483,7 @@
         <v>1000</v>
       </c>
       <c r="D24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E24" s="1">
         <f t="shared" si="12"/>
@@ -1507,7 +1508,7 @@
     </row>
     <row r="25" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A25" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -1519,15 +1520,15 @@
       <c r="I25" s="3"/>
       <c r="J25" s="4">
         <f>SUM(J20:J24)</f>
-        <v>13.072586675</v>
+        <v>12.524927925</v>
       </c>
       <c r="M25" s="1">
         <f>J25</f>
-        <v>13.072586675</v>
+        <v>12.524927925</v>
       </c>
       <c r="N25" s="1">
         <f>J25</f>
-        <v>13.072586675</v>
+        <v>12.524927925</v>
       </c>
     </row>
     <row r="26" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.4">
@@ -1544,25 +1545,25 @@
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A27" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>0</v>
       </c>
       <c r="C27" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E27" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D27" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>25</v>
-      </c>
       <c r="F27" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H27" s="7" t="s">
         <v>1</v>
@@ -1576,7 +1577,7 @@
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B28" s="1">
         <v>19.48</v>
@@ -1585,7 +1586,7 @@
         <v>25</v>
       </c>
       <c r="D28" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E28" s="1">
         <f>10%*SUM(B28, F28)</f>
@@ -1610,49 +1611,49 @@
         <v>1.9883600000000001</v>
       </c>
       <c r="O28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B29" s="1">
-        <v>17.989999999999998</v>
+        <v>13.99</v>
       </c>
       <c r="C29">
         <v>10</v>
       </c>
       <c r="D29" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E29" s="1">
         <f t="shared" ref="E29" si="18">B29*0.1075</f>
-        <v>1.9339249999999999</v>
+        <v>1.503925</v>
       </c>
       <c r="F29" s="1"/>
       <c r="G29" s="1">
         <f t="shared" ref="G29" si="19">B29+E29+F29</f>
-        <v>19.923924999999997</v>
+        <v>15.493925000000001</v>
       </c>
       <c r="H29" s="1">
         <f t="shared" ref="H29" si="20">IF(C29&gt;0, G29/C29, 0)</f>
-        <v>1.9923924999999998</v>
+        <v>1.5493925000000002</v>
       </c>
       <c r="I29">
         <v>1</v>
       </c>
       <c r="J29" s="1">
         <f t="shared" si="17"/>
-        <v>1.9923924999999998</v>
+        <v>1.5493925000000002</v>
       </c>
       <c r="O29" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B30" s="1">
         <v>2.72</v>
@@ -1661,7 +1662,7 @@
         <v>10</v>
       </c>
       <c r="D30" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E30" s="1">
         <f t="shared" ref="E30:E31" si="21">B30*0.1075</f>
@@ -1684,12 +1685,12 @@
         <v>0.30124000000000006</v>
       </c>
       <c r="O30" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B31" s="1">
         <v>8.19</v>
@@ -1698,7 +1699,7 @@
         <v>10</v>
       </c>
       <c r="D31" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E31" s="1">
         <f t="shared" si="21"/>
@@ -1721,7 +1722,7 @@
         <v>0.90704249999999997</v>
       </c>
       <c r="O31" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.4">
@@ -1735,7 +1736,7 @@
       </c>
       <c r="C32">
         <f t="shared" si="22"/>
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D32" t="str">
         <f t="shared" si="22"/>
@@ -1755,23 +1756,23 @@
       </c>
       <c r="H32" s="1">
         <f t="shared" si="22"/>
-        <v>1.0953174999999999</v>
+        <v>0.54765874999999997</v>
       </c>
       <c r="I32">
         <v>-1</v>
       </c>
       <c r="J32" s="1">
         <f>H32*I32</f>
-        <v>-1.0953174999999999</v>
+        <v>-0.54765874999999997</v>
       </c>
       <c r="O32" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="P32" s="5"/>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B33" s="1">
         <v>7.99</v>
@@ -1780,7 +1781,7 @@
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E33" s="1">
         <f t="shared" ref="E33" si="23">B33*0.1075</f>
@@ -1803,12 +1804,12 @@
         <v>1.7697849999999999</v>
       </c>
       <c r="O33" s="5" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B34" s="1">
         <v>1.08</v>
@@ -1817,7 +1818,7 @@
         <v>10</v>
       </c>
       <c r="D34" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E34" s="1">
         <f t="shared" ref="E34" si="26">B34*0.1075</f>
@@ -1840,12 +1841,12 @@
         <v>0.11961000000000002</v>
       </c>
       <c r="O34" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B35" s="1">
         <v>2.02</v>
@@ -1854,7 +1855,7 @@
         <v>10</v>
       </c>
       <c r="D35" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E35" s="1">
         <f t="shared" ref="E35" si="29">B35*0.1075</f>
@@ -1877,12 +1878,12 @@
         <v>0.22371500000000002</v>
       </c>
       <c r="O35" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B36" s="1">
         <v>1.33</v>
@@ -1891,7 +1892,7 @@
         <v>50</v>
       </c>
       <c r="D36" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E36" s="1">
         <f t="shared" ref="E36:E37" si="32">B36*0.1075</f>
@@ -1914,12 +1915,12 @@
         <v>2.9459500000000003E-2</v>
       </c>
       <c r="O36" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B37" s="1">
         <v>0.55000000000000004</v>
@@ -1928,7 +1929,7 @@
         <v>10</v>
       </c>
       <c r="D37" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E37" s="1">
         <f t="shared" si="32"/>
@@ -1951,12 +1952,12 @@
         <v>6.0912500000000001E-2</v>
       </c>
       <c r="O37" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B38" s="1">
         <v>4.79</v>
@@ -1965,19 +1966,19 @@
         <v>20</v>
       </c>
       <c r="D38" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E38" s="1">
-        <f t="shared" ref="E38:E45" si="35">B38*0.1075</f>
+        <f t="shared" ref="E38:E46" si="35">B38*0.1075</f>
         <v>0.51492499999999997</v>
       </c>
       <c r="F38" s="1"/>
       <c r="G38" s="1">
-        <f t="shared" ref="G38:G45" si="36">B38+E38+F38</f>
+        <f t="shared" ref="G38:G46" si="36">B38+E38+F38</f>
         <v>5.3049249999999999</v>
       </c>
       <c r="H38" s="1">
-        <f t="shared" ref="H38:H45" si="37">IF(C38&gt;0, G38/C38, 0)</f>
+        <f t="shared" ref="H38:H46" si="37">IF(C38&gt;0, G38/C38, 0)</f>
         <v>0.26524625000000002</v>
       </c>
       <c r="I38">
@@ -1988,15 +1989,15 @@
         <v>0.26524625000000002</v>
       </c>
       <c r="O38" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="P38" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B39" s="1">
         <v>5.99</v>
@@ -2005,7 +2006,7 @@
         <v>50</v>
       </c>
       <c r="D39" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E39" s="1">
         <f t="shared" si="35"/>
@@ -2024,53 +2025,53 @@
         <v>1</v>
       </c>
       <c r="J39" s="1">
-        <f t="shared" ref="J39:J46" si="38">H39*I39</f>
+        <f t="shared" ref="J39:J47" si="38">H39*I39</f>
         <v>0.1326785</v>
       </c>
       <c r="O39" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B40" s="1">
-        <v>7.95</v>
+        <v>5.66</v>
       </c>
       <c r="C40">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="D40" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E40" s="1">
         <f t="shared" si="35"/>
-        <v>0.85462499999999997</v>
+        <v>0.60845000000000005</v>
       </c>
       <c r="F40" s="1"/>
       <c r="G40" s="1">
         <f t="shared" si="36"/>
-        <v>8.8046249999999997</v>
+        <v>6.2684500000000005</v>
       </c>
       <c r="H40" s="1">
         <f t="shared" si="37"/>
-        <v>0.35218499999999997</v>
+        <v>6.2684500000000004E-2</v>
       </c>
       <c r="I40">
         <v>1</v>
       </c>
       <c r="J40" s="1">
         <f t="shared" si="38"/>
-        <v>0.35218499999999997</v>
+        <v>6.2684500000000004E-2</v>
       </c>
       <c r="O40" s="5" t="s">
-        <v>73</v>
+        <v>107</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B41" s="1">
         <v>25.83</v>
@@ -2079,7 +2080,7 @@
         <v>500</v>
       </c>
       <c r="D41" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E41" s="1">
         <f t="shared" si="35"/>
@@ -2105,7 +2106,7 @@
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B42" s="1">
         <v>0.65</v>
@@ -2114,7 +2115,7 @@
         <v>10</v>
       </c>
       <c r="D42" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E42" s="1">
         <f t="shared" si="35"/>
@@ -2140,221 +2141,247 @@
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
-        <v>87</v>
+        <v>108</v>
       </c>
       <c r="B43" s="1">
-        <v>29.98</v>
+        <v>8.99</v>
       </c>
       <c r="C43">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="D43" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E43" s="1">
         <f t="shared" si="35"/>
-        <v>3.2228500000000002</v>
+        <v>0.96642499999999998</v>
       </c>
       <c r="F43" s="1"/>
       <c r="G43" s="1">
-        <f t="shared" si="36"/>
-        <v>33.202849999999998</v>
+        <f t="shared" ref="G43" si="39">B43+E43+F43</f>
+        <v>9.9564249999999994</v>
       </c>
       <c r="H43" s="1">
-        <f t="shared" si="37"/>
-        <v>0.3320285</v>
+        <f t="shared" ref="H43" si="40">IF(C43&gt;0, G43/C43, 0)</f>
+        <v>0.19912849999999999</v>
       </c>
       <c r="I43">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J43" s="1">
         <f t="shared" si="38"/>
-        <v>1.328114</v>
-      </c>
-      <c r="O43" s="5"/>
+        <v>0.19912849999999999</v>
+      </c>
+      <c r="O43" s="5" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="B44" s="1">
-        <v>5.99</v>
+        <v>29.98</v>
       </c>
       <c r="C44">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="D44" t="s">
         <v>27</v>
       </c>
       <c r="E44" s="1">
         <f t="shared" si="35"/>
-        <v>0.64392499999999997</v>
+        <v>3.2228500000000002</v>
       </c>
       <c r="F44" s="1"/>
       <c r="G44" s="1">
         <f t="shared" si="36"/>
-        <v>6.6339250000000005</v>
+        <v>33.202849999999998</v>
       </c>
       <c r="H44" s="1">
         <f t="shared" si="37"/>
-        <v>6.6339250000000006E-3</v>
+        <v>0.3320285</v>
       </c>
       <c r="I44">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J44" s="1">
-        <f>H44*I44</f>
-        <v>1.3267850000000001E-2</v>
-      </c>
+        <f t="shared" si="38"/>
+        <v>1.328114</v>
+      </c>
+      <c r="O44" s="5"/>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B45" s="1">
-        <v>14.99</v>
+        <v>5.99</v>
       </c>
       <c r="C45">
-        <v>1200</v>
+        <v>1000</v>
       </c>
       <c r="D45" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E45" s="1">
         <f t="shared" si="35"/>
-        <v>1.6114250000000001</v>
+        <v>0.64392499999999997</v>
       </c>
       <c r="F45" s="1"/>
       <c r="G45" s="1">
         <f t="shared" si="36"/>
-        <v>16.601424999999999</v>
+        <v>6.6339250000000005</v>
       </c>
       <c r="H45" s="1">
         <f t="shared" si="37"/>
-        <v>1.3834520833333332E-2</v>
+        <v>6.6339250000000006E-3</v>
       </c>
       <c r="I45">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J45" s="1">
         <f>H45*I45</f>
-        <v>1.3834520833333332E-2</v>
+        <v>1.3267850000000001E-2</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B46" s="1">
-        <v>8.99</v>
+        <v>14.99</v>
       </c>
       <c r="C46">
-        <v>50</v>
+        <v>1200</v>
       </c>
       <c r="D46" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E46" s="1">
-        <f t="shared" ref="E46" si="39">B46*0.1075</f>
-        <v>0.96642499999999998</v>
+        <f t="shared" si="35"/>
+        <v>1.6114250000000001</v>
       </c>
       <c r="F46" s="1"/>
       <c r="G46" s="1">
-        <f t="shared" ref="G46" si="40">B46+E46+F46</f>
+        <f t="shared" si="36"/>
+        <v>16.601424999999999</v>
+      </c>
+      <c r="H46" s="1">
+        <f t="shared" si="37"/>
+        <v>1.3834520833333332E-2</v>
+      </c>
+      <c r="I46">
+        <v>1</v>
+      </c>
+      <c r="J46" s="1">
+        <f>H46*I46</f>
+        <v>1.3834520833333332E-2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A47" t="s">
+        <v>85</v>
+      </c>
+      <c r="B47" s="1">
+        <v>8.99</v>
+      </c>
+      <c r="C47">
+        <v>50</v>
+      </c>
+      <c r="D47" t="s">
+        <v>26</v>
+      </c>
+      <c r="E47" s="1">
+        <f t="shared" ref="E47" si="41">B47*0.1075</f>
+        <v>0.96642499999999998</v>
+      </c>
+      <c r="F47" s="1"/>
+      <c r="G47" s="1">
+        <f t="shared" ref="G47" si="42">B47+E47+F47</f>
         <v>9.9564249999999994</v>
       </c>
-      <c r="H46" s="1">
-        <f t="shared" ref="H46" si="41">IF(C46&gt;0, G46/C46, 0)</f>
+      <c r="H47" s="1">
+        <f t="shared" ref="H47" si="43">IF(C47&gt;0, G47/C47, 0)</f>
         <v>0.19912849999999999</v>
       </c>
-      <c r="I46">
-        <v>1</v>
-      </c>
-      <c r="J46" s="1">
+      <c r="I47">
+        <v>1</v>
+      </c>
+      <c r="J47" s="1">
         <f t="shared" si="38"/>
         <v>0.19912849999999999</v>
       </c>
-      <c r="O46" s="5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A47" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B47" s="3"/>
-      <c r="C47" s="3"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
-      <c r="F47" s="3"/>
-      <c r="G47" s="3"/>
-      <c r="H47" s="3"/>
-      <c r="I47" s="3"/>
-      <c r="J47" s="4">
-        <f>SUM(J28:J46)</f>
-        <v>8.8452819708333319</v>
-      </c>
-      <c r="M47" s="1"/>
-      <c r="N47" s="1">
-        <f>J47</f>
-        <v>8.8452819708333319</v>
-      </c>
-    </row>
-    <row r="48" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="B48" s="1"/>
-      <c r="E48" s="1"/>
-      <c r="F48" s="1"/>
-      <c r="G48" s="1"/>
-      <c r="H48" s="1"/>
-      <c r="J48" s="1"/>
-      <c r="L48" s="7" t="s">
+      <c r="O47" s="5" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A48" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B48" s="3"/>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+      <c r="I48" s="3"/>
+      <c r="J48" s="4">
+        <f>SUM(J28:J47)</f>
+        <v>8.8595687208333302</v>
+      </c>
+      <c r="M48" s="1"/>
+      <c r="N48" s="1">
+        <f>J48</f>
+        <v>8.8595687208333302</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="B49" s="1"/>
+      <c r="E49" s="1"/>
+      <c r="F49" s="1"/>
+      <c r="G49" s="1"/>
+      <c r="H49" s="1"/>
+      <c r="J49" s="1"/>
+      <c r="L49" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="M49" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="N49" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B50" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="M48" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="N48" s="7" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="49" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B49" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C49" s="3"/>
-      <c r="D49" s="3"/>
-      <c r="E49" s="4"/>
-      <c r="F49" s="4"/>
-      <c r="G49" s="4"/>
-      <c r="H49" s="4"/>
-      <c r="I49" s="3"/>
-      <c r="J49" s="4"/>
-      <c r="K49" s="3"/>
-      <c r="L49" s="4">
-        <f>SUM(L3:L48)</f>
-        <v>35.841223606910575</v>
-      </c>
-      <c r="M49" s="4">
-        <f>SUM(M3:M48)</f>
-        <v>17.536535781910569</v>
-      </c>
-      <c r="N49" s="4">
-        <f>SUM(N3:N48)</f>
-        <v>26.381817752743899</v>
-      </c>
-    </row>
-    <row r="50" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="B50" s="1"/>
-      <c r="E50" s="1"/>
-      <c r="F50" s="1"/>
-      <c r="G50" s="1"/>
-      <c r="H50" s="1"/>
-      <c r="J50" s="1"/>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A51" t="s">
-        <v>94</v>
-      </c>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4"/>
+      <c r="G50" s="4"/>
+      <c r="H50" s="4"/>
+      <c r="I50" s="3"/>
+      <c r="J50" s="4"/>
+      <c r="K50" s="3"/>
+      <c r="L50" s="4">
+        <f>SUM(L3:L49)</f>
+        <v>35.728258606910572</v>
+      </c>
+      <c r="M50" s="4">
+        <f>SUM(M3:M49)</f>
+        <v>16.87591203191057</v>
+      </c>
+      <c r="N50" s="4">
+        <f>SUM(N3:N49)</f>
+        <v>25.7354807527439</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.4">
       <c r="B51" s="1"/>
       <c r="E51" s="1"/>
       <c r="F51" s="1"/>
@@ -2364,35 +2391,46 @@
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
-        <v>95</v>
-      </c>
-      <c r="G52" t="s">
-        <v>18</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="B52" s="1"/>
+      <c r="E52" s="1"/>
+      <c r="F52" s="1"/>
+      <c r="G52" s="1"/>
+      <c r="H52" s="1"/>
+      <c r="J52" s="1"/>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
-        <v>96</v>
+        <v>92</v>
+      </c>
+      <c r="G53" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
-        <v>99</v>
+        <v>105</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A58" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2400,14 +2438,14 @@
     <hyperlink ref="O29" r:id="rId1" xr:uid="{394BA01E-496A-4B9E-AF12-01E77921BE0E}"/>
     <hyperlink ref="O30" r:id="rId2" xr:uid="{229E0547-4398-43AE-9042-0D4FDFFB3BD5}"/>
     <hyperlink ref="O22" r:id="rId3" xr:uid="{59869D84-F75A-42B0-B422-BA8AA8AB692E}"/>
-    <hyperlink ref="O40" r:id="rId4" xr:uid="{ED21D2F4-CBE0-426A-A036-B9B33370EF91}"/>
-    <hyperlink ref="O39" r:id="rId5" xr:uid="{916C30C5-416A-439A-9D92-626717DEB750}"/>
-    <hyperlink ref="O20" r:id="rId6" xr:uid="{D1850C95-FE4D-4651-A768-4D4B82A92A51}"/>
-    <hyperlink ref="P21" r:id="rId7" xr:uid="{73F810AA-AEFB-4793-A445-E887A5F2B042}"/>
-    <hyperlink ref="O15" r:id="rId8" xr:uid="{77729D2A-4BC1-468B-9C65-EEFB539A2497}"/>
-    <hyperlink ref="O33" r:id="rId9" xr:uid="{0F1AC341-B54F-4D97-9FD8-521B6BC77D29}"/>
-    <hyperlink ref="O46" r:id="rId10" xr:uid="{B4F36DC8-3A21-4F68-940F-E7861222D837}"/>
-    <hyperlink ref="O8" r:id="rId11" xr:uid="{2073394A-9AF9-4AAC-B9F4-A09AB6C33DED}"/>
+    <hyperlink ref="O39" r:id="rId4" xr:uid="{916C30C5-416A-439A-9D92-626717DEB750}"/>
+    <hyperlink ref="O20" r:id="rId5" xr:uid="{D1850C95-FE4D-4651-A768-4D4B82A92A51}"/>
+    <hyperlink ref="O15" r:id="rId6" xr:uid="{77729D2A-4BC1-468B-9C65-EEFB539A2497}"/>
+    <hyperlink ref="O33" r:id="rId7" xr:uid="{0F1AC341-B54F-4D97-9FD8-521B6BC77D29}"/>
+    <hyperlink ref="O47" r:id="rId8" xr:uid="{B4F36DC8-3A21-4F68-940F-E7861222D837}"/>
+    <hyperlink ref="O8" r:id="rId9" xr:uid="{2073394A-9AF9-4AAC-B9F4-A09AB6C33DED}"/>
+    <hyperlink ref="O43" r:id="rId10" xr:uid="{E068F41A-CE42-4490-B51F-8129D1ECB227}"/>
+    <hyperlink ref="O5" r:id="rId11" xr:uid="{6E17C825-90F1-44D0-95E8-BA1846816186}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="62" fitToWidth="0" orientation="landscape" r:id="rId12"/>
@@ -2431,41 +2469,41 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" t="s">
         <v>40</v>
       </c>
-      <c r="B3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="F3" t="s">
         <v>47</v>
-      </c>
-      <c r="D3" t="s">
-        <v>42</v>
-      </c>
-      <c r="E3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F3" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C5" s="1">
         <v>1.95</v>
@@ -2476,25 +2514,25 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" t="s">
         <v>52</v>
-      </c>
-      <c r="C8" t="s">
-        <v>53</v>
       </c>
       <c r="F8" s="10">
         <v>4</v>
@@ -2502,10 +2540,10 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C9" s="1">
         <v>1.75</v>
@@ -2514,30 +2552,30 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C10" s="1">
         <v>1.33</v>
       </c>
       <c r="D10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E10" s="1">
         <v>0.25</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C11" s="1">
         <v>2.31</v>
@@ -2548,32 +2586,32 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>